<commit_message>
docs: update sprint backlog for J2 perturbation
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-25-sprint-backlog-v1.0.xlsx
+++ b/docs/cadrage/equipe-25-sprint-backlog-v1.0.xlsx
@@ -13,14 +13,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="ys+XiOXYBnzMnIO6NhgObvse86SCAzcspPiqOZCH3Y0="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="LB+Uf5ogXgDAaKcMzI8wXRmmyiPBw4ZyuUTPp96Ic8E="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="174">
   <si>
     <t>A</t>
   </si>
@@ -67,19 +67,19 @@
     <t>Version</t>
   </si>
   <si>
-    <t xml:space="preserve">v1.0 </t>
+    <t>v2</t>
   </si>
   <si>
     <t>Date de remise</t>
   </si>
   <si>
-    <t>29/06/2026 à 14h00</t>
+    <t>30/06/2026 à 17h00</t>
   </si>
   <si>
     <t>Statut</t>
   </si>
   <si>
-    <t>Draft</t>
+    <t>Mis à jour J2</t>
   </si>
   <si>
     <t>💡 Convention de nommage du fichier :</t>
@@ -91,7 +91,7 @@
     <t>SPRINT BACKLOG : SPRINT 1</t>
   </si>
   <si>
-    <t>Lundi PM 14h00 – 18h00 · 28 h-pers · objectif F1+F2 (compte + upload)</t>
+    <t>Lundi PM 14h00 – 18h00 · 24 h-pers · objectif F1+F2 (compte + upload)</t>
   </si>
   <si>
     <t>📋 MÉTADONNÉES DU SPRINT</t>
@@ -226,6 +226,15 @@
     <t>Rizlène</t>
   </si>
   <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>T-01.5</t>
+  </si>
+  <si>
+    <t>Rédiger les critères d’acceptation de l’inscription + vérifier cohérence avec Persona</t>
+  </si>
+  <si>
     <t>US-02</t>
   </si>
   <si>
@@ -250,6 +259,9 @@
     <t>Endpoint POST /api/courses (texte ≥ 200 car) + validation</t>
   </si>
   <si>
+    <t>Done</t>
+  </si>
+  <si>
     <t>T-02.4</t>
   </si>
   <si>
@@ -265,18 +277,57 @@
     <t>Tests pytest + Vitest + ajout README section upload</t>
   </si>
   <si>
-    <t>T-01.5</t>
-  </si>
-  <si>
-    <t>Rédiger les critères d’acceptation de l’inscription + vérifier cohérence avec Persona</t>
-  </si>
-  <si>
     <t>T-02.6</t>
   </si>
   <si>
     <t>Vérifier cohérence Upload cours entre Story Map, Product Backlog et Release Planning</t>
   </si>
   <si>
+    <t>J2</t>
+  </si>
+  <si>
+    <t>T-J2.1</t>
+  </si>
+  <si>
+    <t>Définir le protocole de benchmark : même cours, 5 runs, 3 modèles, p50/p95</t>
+  </si>
+  <si>
+    <t>T-J2.2</t>
+  </si>
+  <si>
+    <t>Benchmarker le modèle actuel llama3.1:8b</t>
+  </si>
+  <si>
+    <t>T-J2.3</t>
+  </si>
+  <si>
+    <t>Benchmarker deux alternatives : llama3.2:3b et phi3:mini</t>
+  </si>
+  <si>
+    <t>T-J2.4</t>
+  </si>
+  <si>
+    <t>Faire noter la qualité subjective /5 par 3 testeurs</t>
+  </si>
+  <si>
+    <t>T-J2.5</t>
+  </si>
+  <si>
+    <t>Rédiger l’ADR J2 : contexte, options, décision, conséquences</t>
+  </si>
+  <si>
+    <t>T-J2.6</t>
+  </si>
+  <si>
+    <t>Bascule du modèle retenu dans la config ou justification de non-action</t>
+  </si>
+  <si>
+    <t>T-J2.7</t>
+  </si>
+  <si>
+    <t>Ré-estimer les stories impactées avant/après perturbation J2</t>
+  </si>
+  <si>
     <t>TOTAL</t>
   </si>
   <si>
@@ -289,9 +340,6 @@
     <t>Tâche pas encore commencée</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
     <t>Tâche en cours (1 seule par personne idéalement)</t>
   </si>
   <si>
@@ -301,9 +349,6 @@
     <t>Tâche bloquée, à remonter en daily</t>
   </si>
   <si>
-    <t>Done</t>
-  </si>
-  <si>
     <t>Tâche terminée et validée</t>
   </si>
   <si>
@@ -493,7 +538,7 @@
     <t>Le Sprint Backlog a été co-construit en Sprint Planning (toutes les voix entendues)</t>
   </si>
   <si>
-    <t>☐ Oui   ✅ Partiel   ☐ Non</t>
+    <t>✅ Oui   ☐ Partiel   ☐ Non</t>
   </si>
   <si>
     <t>Répartition proposée et à valider collectivement en Sprint Planning.</t>
@@ -503,7 +548,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="24">
+  <fonts count="25">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -624,6 +669,11 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -689,7 +739,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border/>
     <border>
       <left style="thin">
@@ -719,11 +769,47 @@
         <color rgb="FF94A3B8"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF666666"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF666666"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF666666"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF666666"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF94A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF94A3B8"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="FF94A3B8"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="50">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -737,63 +823,90 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="2" fillId="2" fontId="14" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="16" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="3" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="4" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="4" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="4" fillId="4" fontId="19" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="4" fontId="20" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="4" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="19" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="6" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="4" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="6" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf borderId="4" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="7" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="2" fillId="7" fontId="20" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="7" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="6" fontId="20" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="4" fillId="5" fontId="19" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="7" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="5" fillId="7" fontId="21" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="7" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="22" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="2" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="24" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2102,7 +2215,7 @@
       <c r="B6" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="12" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2110,7 +2223,7 @@
       <c r="B7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="12" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2118,7 +2231,7 @@
       <c r="B8" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="13" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2126,7 +2239,7 @@
       <c r="B9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="13" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2134,13 +2247,13 @@
       <c r="B10" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="13" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1"/>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="14" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3161,12 +3274,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="16" t="s">
         <v>23</v>
       </c>
     </row>
@@ -3177,66 +3290,66 @@
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="18" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" ht="27.75" customHeight="1">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="18" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="18" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="18" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="9" ht="30.0" customHeight="1">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="18" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="10" ht="81.0" customHeight="1">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="15" t="s">
+      <c r="B10" s="18" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="18" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="15" t="s">
+      <c r="B12" s="18" t="s">
         <v>39</v>
       </c>
     </row>
@@ -3258,7 +3371,7 @@
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="19" t="s">
         <v>44</v>
       </c>
       <c r="B16" s="9" t="s">
@@ -3266,7 +3379,7 @@
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="20" t="s">
         <v>46</v>
       </c>
       <c r="B17" s="9" t="s">
@@ -3275,125 +3388,125 @@
     </row>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C19" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="G19" s="18" t="s">
+      <c r="G19" s="21" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" ht="30.0" customHeight="1">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="E20" s="21">
+      <c r="E20" s="24">
         <v>1.0</v>
       </c>
-      <c r="F20" s="21">
+      <c r="F20" s="24">
         <v>1.0</v>
       </c>
-      <c r="G20" s="20" t="s">
+      <c r="G20" s="23" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="21" ht="30.0" customHeight="1">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="E21" s="21">
+      <c r="E21" s="24">
         <v>2.0</v>
       </c>
-      <c r="F21" s="21">
+      <c r="F21" s="24">
         <v>2.0</v>
       </c>
-      <c r="G21" s="20" t="s">
+      <c r="G21" s="23" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="22" ht="30.0" customHeight="1">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B22" s="19" t="s">
+      <c r="B22" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="20" t="s">
+      <c r="D22" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="24">
         <v>3.0</v>
       </c>
-      <c r="F22" s="21">
+      <c r="F22" s="24">
         <v>3.0</v>
       </c>
-      <c r="G22" s="20" t="s">
+      <c r="G22" s="23" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="23" ht="30.0" customHeight="1">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="C23" s="20" t="s">
+      <c r="C23" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="E23" s="21">
+      <c r="E23" s="24">
         <v>1.0</v>
       </c>
-      <c r="F23" s="21">
+      <c r="F23" s="24">
         <v>1.0</v>
       </c>
-      <c r="G23" s="20" t="s">
-        <v>58</v>
+      <c r="G23" s="25" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="24" ht="30.0" customHeight="1">
-      <c r="A24" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="B24" s="22" t="s">
+      <c r="A24" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="26" t="s">
         <v>69</v>
       </c>
       <c r="C24" s="23" t="s">
@@ -3411,207 +3524,437 @@
       <c r="G24" s="23" t="s">
         <v>58</v>
       </c>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
+      <c r="J24" s="27"/>
+      <c r="K24" s="27"/>
+      <c r="L24" s="27"/>
+      <c r="M24" s="27"/>
+      <c r="N24" s="27"/>
+      <c r="O24" s="27"/>
+      <c r="P24" s="27"/>
+      <c r="Q24" s="27"/>
+      <c r="R24" s="27"/>
+      <c r="S24" s="27"/>
+      <c r="T24" s="27"/>
+      <c r="U24" s="27"/>
+      <c r="V24" s="27"/>
+      <c r="W24" s="27"/>
+      <c r="X24" s="27"/>
+      <c r="Y24" s="27"/>
+      <c r="Z24" s="27"/>
     </row>
     <row r="25" ht="30.0" customHeight="1">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B25" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C25" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="D25" s="29" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" s="30">
+        <v>1.0</v>
+      </c>
+      <c r="F25" s="30">
+        <v>1.0</v>
+      </c>
+      <c r="G25" s="29" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" ht="30.0" customHeight="1">
+      <c r="A26" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="D26" s="29" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" s="30">
+        <v>3.0</v>
+      </c>
+      <c r="F26" s="30">
+        <v>3.0</v>
+      </c>
+      <c r="G26" s="29" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="27" ht="30.0" customHeight="1">
+      <c r="A27" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" s="30">
+        <v>1.0</v>
+      </c>
+      <c r="F27" s="31">
+        <v>0.0</v>
+      </c>
+      <c r="G27" s="32" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" ht="30.0" customHeight="1">
+      <c r="A28" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="C28" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="E28" s="30">
+        <v>3.0</v>
+      </c>
+      <c r="F28" s="30">
+        <v>3.0</v>
+      </c>
+      <c r="G28" s="29" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" ht="30.0" customHeight="1">
+      <c r="A29" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C29" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="D29" s="29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" s="30">
+        <v>1.0</v>
+      </c>
+      <c r="F29" s="31">
+        <v>0.0</v>
+      </c>
+      <c r="G29" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="H29" s="33"/>
+      <c r="I29" s="33"/>
+      <c r="J29" s="33"/>
+      <c r="K29" s="33"/>
+      <c r="L29" s="33"/>
+      <c r="M29" s="33"/>
+      <c r="N29" s="33"/>
+      <c r="O29" s="33"/>
+      <c r="P29" s="33"/>
+      <c r="Q29" s="33"/>
+      <c r="R29" s="33"/>
+      <c r="S29" s="33"/>
+      <c r="T29" s="33"/>
+      <c r="U29" s="33"/>
+      <c r="V29" s="33"/>
+      <c r="W29" s="33"/>
+      <c r="X29" s="33"/>
+      <c r="Y29" s="33"/>
+      <c r="Z29" s="33"/>
+    </row>
+    <row r="30" ht="30.0" customHeight="1">
+      <c r="A30" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B30" s="34" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="29" t="s">
+        <v>61</v>
+      </c>
+      <c r="E30" s="30">
+        <v>1.0</v>
+      </c>
+      <c r="F30" s="30">
+        <v>1.0</v>
+      </c>
+      <c r="G30" s="29" t="s">
+        <v>58</v>
+      </c>
+      <c r="H30" s="33"/>
+      <c r="I30" s="33"/>
+      <c r="J30" s="33"/>
+      <c r="K30" s="33"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="33"/>
+      <c r="N30" s="33"/>
+      <c r="O30" s="33"/>
+      <c r="P30" s="33"/>
+      <c r="Q30" s="33"/>
+      <c r="R30" s="33"/>
+      <c r="S30" s="33"/>
+      <c r="T30" s="33"/>
+      <c r="U30" s="33"/>
+      <c r="V30" s="33"/>
+      <c r="W30" s="33"/>
+      <c r="X30" s="33"/>
+      <c r="Y30" s="33"/>
+      <c r="Z30" s="33"/>
+    </row>
+    <row r="31" ht="30.0" customHeight="1">
+      <c r="A31" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B31" s="35" t="s">
+        <v>88</v>
+      </c>
+      <c r="C31" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="E31" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F31" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="G31" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="H31" s="33"/>
+      <c r="I31" s="33"/>
+      <c r="J31" s="33"/>
+      <c r="K31" s="33"/>
+      <c r="L31" s="33"/>
+      <c r="M31" s="33"/>
+      <c r="N31" s="33"/>
+      <c r="O31" s="33"/>
+      <c r="P31" s="33"/>
+      <c r="Q31" s="33"/>
+      <c r="R31" s="33"/>
+      <c r="S31" s="33"/>
+      <c r="T31" s="33"/>
+      <c r="U31" s="33"/>
+      <c r="V31" s="33"/>
+      <c r="W31" s="33"/>
+      <c r="X31" s="33"/>
+      <c r="Y31" s="33"/>
+      <c r="Z31" s="33"/>
+    </row>
+    <row r="32" ht="30.0" customHeight="1">
+      <c r="A32" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="C32" s="32" t="s">
+        <v>91</v>
+      </c>
+      <c r="D32" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="E32" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F32" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="G32" s="32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="33" ht="30.0" customHeight="1">
+      <c r="A33" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B33" s="35" t="s">
+        <v>92</v>
+      </c>
+      <c r="C33" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="D33" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" s="31">
+        <v>2.0</v>
+      </c>
+      <c r="F33" s="31">
+        <v>2.0</v>
+      </c>
+      <c r="G33" s="32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="34" ht="30.0" customHeight="1">
+      <c r="A34" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B34" s="35" t="s">
+        <v>94</v>
+      </c>
+      <c r="C34" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="D34" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="E34" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F34" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="G34" s="32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="35" ht="30.0" customHeight="1">
+      <c r="A35" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B35" s="35" t="s">
+        <v>96</v>
+      </c>
+      <c r="C35" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="D35" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="E35" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F35" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="G35" s="32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="36" ht="30.0" customHeight="1">
+      <c r="A36" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B36" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="C36" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="D36" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="E36" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F36" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="G36" s="32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="37" ht="30.0" customHeight="1">
+      <c r="A37" s="35" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37" s="35" t="s">
+        <v>100</v>
+      </c>
+      <c r="C37" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="D37" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="E37" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F37" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="G37" s="32" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="38" ht="14.25" customHeight="1">
+      <c r="A38" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="B38" s="37"/>
+      <c r="C38" s="38" t="s">
+        <v>103</v>
+      </c>
+      <c r="D38" s="37"/>
+      <c r="E38" s="39">
+        <v>26.0</v>
+      </c>
+      <c r="F38" s="39">
+        <v>24.0</v>
+      </c>
+      <c r="G38" s="37"/>
+    </row>
+    <row r="39" ht="14.25" customHeight="1"/>
+    <row r="40" ht="14.25" customHeight="1">
+      <c r="A40" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" ht="14.25" customHeight="1">
+      <c r="A41" s="40" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" s="9" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="42" ht="14.25" customHeight="1">
+      <c r="A42" s="41" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="C25" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="D25" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="E25" s="24">
-        <v>3.0</v>
-      </c>
-      <c r="F25" s="24">
-        <v>3.0</v>
-      </c>
-      <c r="G25" s="23" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="26" ht="30.0" customHeight="1">
-      <c r="A26" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="C26" s="23" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E26" s="24">
-        <v>1.0</v>
-      </c>
-      <c r="F26" s="24">
-        <v>1.0</v>
-      </c>
-      <c r="G26" s="23" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="27" ht="30.0" customHeight="1">
-      <c r="A27" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="B27" s="22" t="s">
-        <v>76</v>
-      </c>
-      <c r="C27" s="23" t="s">
-        <v>77</v>
-      </c>
-      <c r="D27" s="23" t="s">
-        <v>78</v>
-      </c>
-      <c r="E27" s="24">
-        <v>3.0</v>
-      </c>
-      <c r="F27" s="24">
-        <v>3.0</v>
-      </c>
-      <c r="G27" s="23" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="28" ht="30.0" customHeight="1">
-      <c r="A28" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="22" t="s">
+      <c r="B42" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="43" ht="14.25" customHeight="1">
+      <c r="A43" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="B43" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="44" ht="14.25" customHeight="1">
+      <c r="A44" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="C28" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="D28" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E28" s="24">
-        <v>1.0</v>
-      </c>
-      <c r="F28" s="24">
-        <v>1.0</v>
-      </c>
-      <c r="G28" s="23" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" ht="30.0" customHeight="1">
-      <c r="A29" s="25" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="25" t="s">
-        <v>81</v>
-      </c>
-      <c r="C29" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="D29" s="26" t="s">
-        <v>57</v>
-      </c>
-      <c r="E29" s="27">
-        <v>1.0</v>
-      </c>
-      <c r="F29" s="27">
-        <v>1.0</v>
-      </c>
-      <c r="G29" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="30" ht="30.0" customHeight="1">
-      <c r="A30" s="25" t="s">
-        <v>68</v>
-      </c>
-      <c r="B30" s="25" t="s">
-        <v>83</v>
-      </c>
-      <c r="C30" s="26" t="s">
-        <v>84</v>
-      </c>
-      <c r="D30" s="26" t="s">
-        <v>61</v>
-      </c>
-      <c r="E30" s="27">
-        <v>1.0</v>
-      </c>
-      <c r="F30" s="27">
-        <v>1.0</v>
-      </c>
-      <c r="G30" s="26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="31" ht="14.25" customHeight="1">
-      <c r="A31" s="28" t="s">
-        <v>85</v>
-      </c>
-      <c r="B31" s="29"/>
-      <c r="C31" s="30" t="s">
-        <v>86</v>
-      </c>
-      <c r="D31" s="29"/>
-      <c r="E31" s="28">
-        <v>18.0</v>
-      </c>
-      <c r="F31" s="28">
-        <v>18.0</v>
-      </c>
-      <c r="G31" s="29"/>
-    </row>
-    <row r="32" ht="14.25" customHeight="1"/>
-    <row r="33" ht="14.25" customHeight="1">
-      <c r="A33" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="34" ht="14.25" customHeight="1">
-      <c r="A34" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="35" ht="14.25" customHeight="1">
-      <c r="A35" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="36" ht="14.25" customHeight="1">
-      <c r="A36" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="37" ht="14.25" customHeight="1">
-      <c r="A37" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="38" ht="14.25" customHeight="1"/>
-    <row r="39" ht="14.25" customHeight="1"/>
-    <row r="40" ht="14.25" customHeight="1"/>
-    <row r="41" ht="14.25" customHeight="1"/>
-    <row r="42" ht="14.25" customHeight="1"/>
-    <row r="43" ht="14.25" customHeight="1"/>
-    <row r="44" ht="14.25" customHeight="1"/>
+      <c r="B44" s="9" t="s">
+        <v>109</v>
+      </c>
+    </row>
     <row r="45" ht="14.25" customHeight="1"/>
     <row r="46" ht="14.25" customHeight="1"/>
     <row r="47" ht="14.25" customHeight="1"/>
@@ -4569,6 +4912,13 @@
     <row r="999" ht="14.25" customHeight="1"/>
     <row r="1000" ht="14.25" customHeight="1"/>
     <row r="1001" ht="14.25" customHeight="1"/>
+    <row r="1002" ht="14.25" customHeight="1"/>
+    <row r="1003" ht="14.25" customHeight="1"/>
+    <row r="1004" ht="14.25" customHeight="1"/>
+    <row r="1005" ht="14.25" customHeight="1"/>
+    <row r="1006" ht="14.25" customHeight="1"/>
+    <row r="1007" ht="14.25" customHeight="1"/>
+    <row r="1008" ht="14.25" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -4592,173 +4942,173 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="13" t="s">
-        <v>95</v>
+      <c r="A1" s="15" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1"/>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1"/>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="18" t="s">
-        <v>101</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>102</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>103</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>104</v>
-      </c>
-      <c r="E7" s="18" t="s">
-        <v>105</v>
+      <c r="A7" s="42" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="42" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="42" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" s="42" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
-      <c r="A8" s="33" t="s">
-        <v>106</v>
-      </c>
-      <c r="B8" s="34">
+      <c r="A8" s="43" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" s="44">
         <v>18.0</v>
       </c>
-      <c r="C8" s="34">
+      <c r="C8" s="44">
         <v>18.0</v>
       </c>
-      <c r="D8" s="34">
+      <c r="D8" s="44">
         <v>0.0</v>
       </c>
-      <c r="E8" s="15" t="s">
-        <v>107</v>
+      <c r="E8" s="18" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="9" ht="24.75" customHeight="1">
-      <c r="A9" s="33" t="s">
-        <v>108</v>
-      </c>
-      <c r="B9" s="34">
+      <c r="A9" s="43" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="44">
         <v>13.5</v>
       </c>
-      <c r="C9" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="34"/>
-      <c r="E9" s="15" t="s">
-        <v>110</v>
+      <c r="C9" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="44"/>
+      <c r="E9" s="18" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="10" ht="24.75" customHeight="1">
-      <c r="A10" s="33" t="s">
-        <v>111</v>
-      </c>
-      <c r="B10" s="34">
+      <c r="A10" s="43" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="44">
         <v>9.0</v>
       </c>
-      <c r="C10" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="D10" s="34"/>
-      <c r="E10" s="15" t="s">
-        <v>112</v>
+      <c r="C10" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="D10" s="44"/>
+      <c r="E10" s="18" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="11" ht="24.75" customHeight="1">
-      <c r="A11" s="33" t="s">
-        <v>113</v>
-      </c>
-      <c r="B11" s="34">
+      <c r="A11" s="43" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" s="44">
         <v>4.5</v>
       </c>
-      <c r="C11" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="D11" s="34"/>
-      <c r="E11" s="15" t="s">
-        <v>114</v>
+      <c r="C11" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="D11" s="44"/>
+      <c r="E11" s="18" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="12" ht="24.75" customHeight="1">
-      <c r="A12" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="B12" s="34">
+      <c r="A12" s="43" t="s">
+        <v>130</v>
+      </c>
+      <c r="B12" s="44">
         <v>0.0</v>
       </c>
-      <c r="C12" s="34" t="s">
-        <v>109</v>
-      </c>
-      <c r="D12" s="34"/>
-      <c r="E12" s="15" t="s">
-        <v>116</v>
+      <c r="C12" s="44" t="s">
+        <v>124</v>
+      </c>
+      <c r="D12" s="44"/>
+      <c r="E12" s="18" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1"/>
     <row r="14" ht="14.25" customHeight="1"/>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="A18" s="16" t="s">
-        <v>120</v>
+      <c r="A18" s="19" t="s">
+        <v>135</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="32" t="s">
-        <v>122</v>
+      <c r="A19" s="41" t="s">
+        <v>137</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" s="16" t="s">
-        <v>124</v>
+      <c r="A20" s="19" t="s">
+        <v>139</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" s="17" t="s">
-        <v>126</v>
+      <c r="A21" s="20" t="s">
+        <v>141</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1"/>
@@ -5765,135 +6115,135 @@
     <row r="1" ht="14.25" customHeight="1"/>
     <row r="2" ht="14.25" customHeight="1">
       <c r="B2" s="2" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="B3" s="9" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1"/>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="18"/>
-      <c r="B5" s="18" t="s">
-        <v>130</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="D5" s="35" t="s">
-        <v>132</v>
+      <c r="A5" s="42"/>
+      <c r="B5" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="C5" s="42" t="s">
+        <v>146</v>
+      </c>
+      <c r="D5" s="45" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="6" ht="30.0" customHeight="1">
-      <c r="B6" s="36" t="s">
-        <v>133</v>
-      </c>
-      <c r="C6" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="D6" s="36" t="s">
-        <v>135</v>
+      <c r="B6" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="47" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="46" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="7" ht="30.0" customHeight="1">
-      <c r="B7" s="36" t="s">
-        <v>136</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>137</v>
-      </c>
-      <c r="D7" s="36" t="s">
-        <v>138</v>
+      <c r="B7" s="46" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="47" t="s">
+        <v>152</v>
+      </c>
+      <c r="D7" s="46" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="8" ht="30.0" customHeight="1">
-      <c r="B8" s="36" t="s">
-        <v>139</v>
-      </c>
-      <c r="C8" s="37" t="s">
-        <v>140</v>
-      </c>
-      <c r="D8" s="36" t="s">
-        <v>141</v>
+      <c r="B8" s="46" t="s">
+        <v>154</v>
+      </c>
+      <c r="C8" s="47" t="s">
+        <v>155</v>
+      </c>
+      <c r="D8" s="46" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="9" ht="30.0" customHeight="1">
-      <c r="B9" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="C9" s="37" t="s">
-        <v>137</v>
-      </c>
-      <c r="D9" s="36" t="s">
-        <v>143</v>
+      <c r="B9" s="46" t="s">
+        <v>157</v>
+      </c>
+      <c r="C9" s="47" t="s">
+        <v>152</v>
+      </c>
+      <c r="D9" s="46" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="10" ht="30.0" customHeight="1">
-      <c r="B10" s="36" t="s">
-        <v>144</v>
-      </c>
-      <c r="C10" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="D10" s="36" t="s">
-        <v>146</v>
+      <c r="B10" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="C10" s="47" t="s">
+        <v>160</v>
+      </c>
+      <c r="D10" s="46" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="11" ht="30.0" customHeight="1">
-      <c r="B11" s="36" t="s">
-        <v>147</v>
-      </c>
-      <c r="C11" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="D11" s="38" t="s">
-        <v>148</v>
+      <c r="B11" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" s="47" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="12" ht="30.0" customHeight="1">
-      <c r="B12" s="36" t="s">
-        <v>149</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="D12" s="36" t="s">
-        <v>150</v>
+      <c r="B12" s="46" t="s">
+        <v>164</v>
+      </c>
+      <c r="C12" s="47" t="s">
+        <v>160</v>
+      </c>
+      <c r="D12" s="46" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="13" ht="30.0" customHeight="1">
-      <c r="B13" s="36" t="s">
-        <v>151</v>
-      </c>
-      <c r="C13" s="37" t="s">
-        <v>152</v>
-      </c>
-      <c r="D13" s="36" t="s">
-        <v>153</v>
+      <c r="B13" s="46" t="s">
+        <v>166</v>
+      </c>
+      <c r="C13" s="47" t="s">
+        <v>167</v>
+      </c>
+      <c r="D13" s="46" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="14" ht="30.0" customHeight="1">
-      <c r="B14" s="36" t="s">
-        <v>154</v>
-      </c>
-      <c r="C14" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="D14" s="36" t="s">
-        <v>155</v>
+      <c r="B14" s="46" t="s">
+        <v>169</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>160</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="15" ht="30.0" customHeight="1">
-      <c r="B15" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="C15" s="37" t="s">
-        <v>157</v>
-      </c>
-      <c r="D15" s="36" t="s">
-        <v>158</v>
+      <c r="B15" s="46" t="s">
+        <v>171</v>
+      </c>
+      <c r="C15" s="49" t="s">
+        <v>172</v>
+      </c>
+      <c r="D15" s="46" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
docs: update sprint backlog for J4
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-25-sprint-backlog-v1.0.xlsx
+++ b/docs/cadrage/equipe-25-sprint-backlog-v1.0.xlsx
@@ -5,22 +5,23 @@
   <sheets>
     <sheet state="visible" name="Garde" sheetId="1" r:id="rId4"/>
     <sheet state="visible" name="Identification" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="Sprint 1" sheetId="3" r:id="rId6"/>
-    <sheet state="visible" name="Burndown Sprint 1" sheetId="4" r:id="rId7"/>
-    <sheet state="visible" name="Auto-évaluation" sheetId="5" r:id="rId8"/>
+    <sheet state="visible" name="Historique sprint backlog" sheetId="3" r:id="rId6"/>
+    <sheet state="visible" name="Next sprint backlog J4" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="Burndown Sprint 1" sheetId="5" r:id="rId8"/>
+    <sheet state="visible" name="Auto-évaluation" sheetId="6" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="OkMD2GZErxh/c7I+mAF6DHtZZBs4i2A6YDI6VlOZ/sU="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId10" roundtripDataChecksum="v4d6Nhb+IgKqBLIhJ1avFvi2+EQopLctnCsrVsEWyC0="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="227">
   <si>
     <t>A</t>
   </si>
@@ -61,25 +62,25 @@
     <t>Sprint concerné</t>
   </si>
   <si>
-    <t>Sprint 1</t>
+    <t>Sprint 7</t>
   </si>
   <si>
     <t>Version</t>
   </si>
   <si>
-    <t>v3</t>
+    <t>v4</t>
   </si>
   <si>
     <t>Date de remise</t>
   </si>
   <si>
-    <t>30/06/2026 à 17h00</t>
+    <t>02/07/2026 à 14h00</t>
   </si>
   <si>
     <t>Statut</t>
   </si>
   <si>
-    <t>Mis à jour J3</t>
+    <t>Mis à jour J4</t>
   </si>
   <si>
     <t>💡 Convention de nommage du fichier :</t>
@@ -88,10 +89,10 @@
     <t>equipe-XX-nom-document-vY.Z.xlsx  (ex. equipe-03-product-backlog-v1.0.xlsx)</t>
   </si>
   <si>
-    <t>SPRINT BACKLOG : SPRINT 1</t>
-  </si>
-  <si>
-    <t>Lundi PM 14h00 – 18h00 · 24 h-pers · objectif F1+F2 (compte + upload)</t>
+    <t>SPRINT BACKLOG : Historique sprint backlog</t>
+  </si>
+  <si>
+    <t>Historique cumulé des tâches Sprint 1 + perturbations J2/J3/J4</t>
   </si>
   <si>
     <t>📋 MÉTADONNÉES DU SPRINT</t>
@@ -100,10 +101,13 @@
     <t>Numéro de sprint</t>
   </si>
   <si>
+    <t>Sprint 1 à Sprint 7</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
-    <t>Lundi 26/06/2026 ], 14h00 à  18h00 (4 h)</t>
+    <t>02/07/2026 , 14h00 à  18h00</t>
   </si>
   <si>
     <t>Équipe (n personnes)</t>
@@ -121,13 +125,13 @@
     <t>Vélocité cible (SP)</t>
   </si>
   <si>
-    <t>8 à 10 SP (US-01 = 3 SP, US-02 = 5 SP)</t>
+    <t>Historique cumulé — estimations mises à jour après J2/J3/J4</t>
   </si>
   <si>
     <t>Objectif sprint</t>
   </si>
   <si>
-    <t>Démarrer les features F1 (inscription) et F2 (upload cours), démontrable en Sprint Review 18h</t>
+    <t>Conserver l’historique des tâches réalisées, en cours et ajoutées suite aux perturbations J2, J3 et J4.</t>
   </si>
   <si>
     <t>Scrum Master</t>
@@ -379,10 +383,100 @@
     <t>Mettre à jour la DoD sécurité / vérifier conformité avec les critères d’acceptation J3</t>
   </si>
   <si>
+    <t>J4-a11y</t>
+  </si>
+  <si>
+    <t>T-J4.1</t>
+  </si>
+  <si>
+    <t>Réaliser un audit RGAA rapide : contrastes, navigation clavier, focus visible</t>
+  </si>
+  <si>
+    <t>T-J4.2</t>
+  </si>
+  <si>
+    <t>Corriger les contrastes et rendre les boutons/formulaires accessibles clavier</t>
+  </si>
+  <si>
+    <t>T-J4.3</t>
+  </si>
+  <si>
+    <t>Ajouter labels, alt text et structure sémantique pour lecteur d’écran</t>
+  </si>
+  <si>
+    <t>J4-i18n</t>
+  </si>
+  <si>
+    <t>T-J4.4</t>
+  </si>
+  <si>
+    <t>Externaliser les textes de l’interface dans des fichiers de langue FR/EN/ES</t>
+  </si>
+  <si>
+    <t>T-J4.5</t>
+  </si>
+  <si>
+    <t>Ajouter un sélecteur de langue dans l’interface</t>
+  </si>
+  <si>
+    <t>T-J4.6</t>
+  </si>
+  <si>
+    <t>Ajouter un paramètre de langue pour que le LLM génère les quiz dans la langue choisie</t>
+  </si>
+  <si>
+    <t>J4-scale</t>
+  </si>
+  <si>
+    <t>T-J4.7</t>
+  </si>
+  <si>
+    <t>Réaliser un test de charge simple sur génération de quiz et navigation</t>
+  </si>
+  <si>
+    <t>T-J4.8</t>
+  </si>
+  <si>
+    <t>Proposer une architecture scalable : cache, file d’attente LLM, autoscaling</t>
+  </si>
+  <si>
+    <t>T-J4.9</t>
+  </si>
+  <si>
+    <t>Ajouter un fournisseur LLM de secours ou rédiger un ADR de résilience</t>
+  </si>
+  <si>
+    <t>J4-risk</t>
+  </si>
+  <si>
+    <t>T-J4.10</t>
+  </si>
+  <si>
+    <t>Relier les risques prioritaires à des actions préventives dans le backlog</t>
+  </si>
+  <si>
+    <t>J4-pilotage</t>
+  </si>
+  <si>
+    <t>T-J4.11</t>
+  </si>
+  <si>
+    <t>Mettre à jour burndown et burnup avec le nouveau périmètre J4</t>
+  </si>
+  <si>
+    <t>J4-doc</t>
+  </si>
+  <si>
+    <t>T-J4.12</t>
+  </si>
+  <si>
+    <t>Vérifier cohérence entre personas, story map, product backlog et release planning</t>
+  </si>
+  <si>
     <t>TOTAL</t>
   </si>
   <si>
-    <t>36 h estimées après perturbations J2 + J3 · capacité initiale 24 h-pers · dépassement de 12 h à arbitrer en équipe</t>
+    <t>36 h estimées après perturbations J2 + J3 + J4 · capacité initiale 24 h-pers · dépassement de 12 h à arbitrer en équipe</t>
   </si>
   <si>
     <t>📌 STATUTS</t>
@@ -401,6 +495,21 @@
   </si>
   <si>
     <t>Tâche terminée et validée</t>
+  </si>
+  <si>
+    <t>SPRINT BACKLOG : NEXT SPRINT BACKLOG · SPRINT 7</t>
+  </si>
+  <si>
+    <t>Jeudi PM 14h00 – 18h00 · objectif J4 : RGAA + i18n + scalabilité + risques + pilotage</t>
+  </si>
+  <si>
+    <t>20 à 25 SP estimés sur les axes RGAA, i18n, scalabilité et risques</t>
+  </si>
+  <si>
+    <t>Préparer le passage à l’échelle d’EduTutor IA : accessibilité RGAA, internationalisation, scalabilité, analyse de risques et pilotage burndown/burnup.</t>
+  </si>
+  <si>
+    <t>25 h estimées pour le next sprint · périmètre J4 : accessibilité RGAA, i18n, scalabilité, risques et pilotage</t>
   </si>
   <si>
     <t>BURNDOWN : SPRINT 1</t>
@@ -599,7 +708,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="25">
+  <fonts count="27">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -723,6 +832,15 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF1E1B4B"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF1E1B4B"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11.0"/>
@@ -885,7 +1003,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="63">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -907,11 +1025,16 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="2" fillId="2" fontId="14" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -972,16 +1095,32 @@
     <xf borderId="6" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
+    <xf borderId="6" fillId="5" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="5" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="6" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="7" fillId="7" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="7" fillId="7" fontId="21" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="7" fontId="23" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="7" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="22" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="24" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="25" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -991,17 +1130,17 @@
     <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="24" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="26" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1029,6 +1168,10 @@
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -2319,7 +2462,7 @@
       <c r="B7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="13" t="s">
         <v>13</v>
       </c>
     </row>
@@ -3369,7 +3512,7 @@
     <col customWidth="1" min="8" max="26" width="8.86"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
+    <row r="1" ht="23.25" customHeight="1">
       <c r="A1" s="15" t="s">
         <v>22</v>
       </c>
@@ -3390,847 +3533,1146 @@
         <v>25</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" ht="27.75" customHeight="1">
       <c r="A6" s="17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
       <c r="A7" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="18" t="s">
         <v>29</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
       <c r="A8" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="18" t="s">
         <v>31</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="9" ht="30.0" customHeight="1">
       <c r="A9" s="17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" ht="81.0" customHeight="1">
       <c r="A10" s="17" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
       <c r="A11" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="18" t="s">
         <v>37</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
       <c r="A12" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B12" s="18" t="s">
         <v>39</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1"/>
     <row r="14" ht="14.25" customHeight="1">
       <c r="A14" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="A16" s="19" t="s">
-        <v>44</v>
+      <c r="A16" s="20" t="s">
+        <v>45</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" s="20" t="s">
-        <v>46</v>
+      <c r="A17" s="21" t="s">
+        <v>47</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="B19" s="21" t="s">
+      <c r="A19" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="B19" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="21" t="s">
+      <c r="C19" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="21" t="s">
+      <c r="D19" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="F19" s="21" t="s">
+      <c r="E19" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="G19" s="21" t="s">
+      <c r="F19" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="22" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" ht="30.0" customHeight="1">
-      <c r="A20" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B20" s="22" t="s">
+      <c r="A20" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="B20" s="23" t="s">
         <v>56</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="C20" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="E20" s="24">
+      <c r="D20" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" s="25">
         <v>1.0</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="25">
         <v>1.0</v>
       </c>
-      <c r="G20" s="23" t="s">
+      <c r="G20" s="24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" ht="30.0" customHeight="1">
+      <c r="A21" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>61</v>
+      </c>
+      <c r="D21" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="E21" s="25">
+        <v>2.0</v>
+      </c>
+      <c r="F21" s="25">
+        <v>2.0</v>
+      </c>
+      <c r="G21" s="24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" ht="30.0" customHeight="1">
+      <c r="A22" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>64</v>
+      </c>
+      <c r="D22" s="24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" s="25">
+        <v>3.0</v>
+      </c>
+      <c r="F22" s="25">
+        <v>3.0</v>
+      </c>
+      <c r="G22" s="24" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" ht="30.0" customHeight="1">
+      <c r="A23" s="23" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23" s="24" t="s">
+        <v>68</v>
+      </c>
+      <c r="E23" s="25">
+        <v>1.0</v>
+      </c>
+      <c r="F23" s="25">
+        <v>1.0</v>
+      </c>
+      <c r="G23" s="26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="24" ht="30.0" customHeight="1">
+      <c r="A24" s="27" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="24" t="s">
+        <v>71</v>
+      </c>
+      <c r="D24" s="24" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="21" ht="30.0" customHeight="1">
-      <c r="A21" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B21" s="22" t="s">
+      <c r="E24" s="25">
+        <v>1.0</v>
+      </c>
+      <c r="F24" s="25">
+        <v>1.0</v>
+      </c>
+      <c r="G24" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="C21" s="23" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="23" t="s">
-        <v>61</v>
-      </c>
-      <c r="E21" s="24">
+      <c r="H24" s="28"/>
+      <c r="I24" s="28"/>
+      <c r="J24" s="28"/>
+      <c r="K24" s="28"/>
+      <c r="L24" s="28"/>
+      <c r="M24" s="28"/>
+      <c r="N24" s="28"/>
+      <c r="O24" s="28"/>
+      <c r="P24" s="28"/>
+      <c r="Q24" s="28"/>
+      <c r="R24" s="28"/>
+      <c r="S24" s="28"/>
+      <c r="T24" s="28"/>
+      <c r="U24" s="28"/>
+      <c r="V24" s="28"/>
+      <c r="W24" s="28"/>
+      <c r="X24" s="28"/>
+      <c r="Y24" s="28"/>
+      <c r="Z24" s="28"/>
+    </row>
+    <row r="25" ht="30.0" customHeight="1">
+      <c r="A25" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="B25" s="29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="30" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" s="30" t="s">
+        <v>58</v>
+      </c>
+      <c r="E25" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F25" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="G25" s="30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" ht="30.0" customHeight="1">
+      <c r="A26" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" s="29" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="30" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" s="30" t="s">
+        <v>77</v>
+      </c>
+      <c r="E26" s="31">
+        <v>3.0</v>
+      </c>
+      <c r="F26" s="31">
+        <v>3.0</v>
+      </c>
+      <c r="G26" s="30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" ht="30.0" customHeight="1">
+      <c r="A27" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="B27" s="29" t="s">
+        <v>78</v>
+      </c>
+      <c r="C27" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E27" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F27" s="32">
+        <v>0.0</v>
+      </c>
+      <c r="G27" s="33" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" ht="30.0" customHeight="1">
+      <c r="A28" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" s="29" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="D28" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="E28" s="31">
+        <v>3.0</v>
+      </c>
+      <c r="F28" s="31">
+        <v>3.0</v>
+      </c>
+      <c r="G28" s="30" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" ht="30.0" customHeight="1">
+      <c r="A29" s="29" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>85</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E29" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F29" s="32">
+        <v>0.0</v>
+      </c>
+      <c r="G29" s="33" t="s">
+        <v>80</v>
+      </c>
+      <c r="H29" s="34"/>
+      <c r="I29" s="34"/>
+      <c r="J29" s="34"/>
+      <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
+      <c r="M29" s="34"/>
+      <c r="N29" s="34"/>
+      <c r="O29" s="34"/>
+      <c r="P29" s="34"/>
+      <c r="Q29" s="34"/>
+      <c r="R29" s="34"/>
+      <c r="S29" s="34"/>
+      <c r="T29" s="34"/>
+      <c r="U29" s="34"/>
+      <c r="V29" s="34"/>
+      <c r="W29" s="34"/>
+      <c r="X29" s="34"/>
+      <c r="Y29" s="34"/>
+      <c r="Z29" s="34"/>
+    </row>
+    <row r="30" ht="30.0" customHeight="1">
+      <c r="A30" s="35" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" s="35" t="s">
+        <v>86</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="D30" s="30" t="s">
+        <v>62</v>
+      </c>
+      <c r="E30" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="F30" s="31">
+        <v>1.0</v>
+      </c>
+      <c r="G30" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="H30" s="34"/>
+      <c r="I30" s="34"/>
+      <c r="J30" s="34"/>
+      <c r="K30" s="34"/>
+      <c r="L30" s="34"/>
+      <c r="M30" s="34"/>
+      <c r="N30" s="34"/>
+      <c r="O30" s="34"/>
+      <c r="P30" s="34"/>
+      <c r="Q30" s="34"/>
+      <c r="R30" s="34"/>
+      <c r="S30" s="34"/>
+      <c r="T30" s="34"/>
+      <c r="U30" s="34"/>
+      <c r="V30" s="34"/>
+      <c r="W30" s="34"/>
+      <c r="X30" s="34"/>
+      <c r="Y30" s="34"/>
+      <c r="Z30" s="34"/>
+    </row>
+    <row r="31" ht="30.0" customHeight="1">
+      <c r="A31" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B31" s="36" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="33" t="s">
+        <v>90</v>
+      </c>
+      <c r="D31" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="E31" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="F31" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="G31" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="H31" s="34"/>
+      <c r="I31" s="34"/>
+      <c r="J31" s="34"/>
+      <c r="K31" s="34"/>
+      <c r="L31" s="34"/>
+      <c r="M31" s="34"/>
+      <c r="N31" s="34"/>
+      <c r="O31" s="34"/>
+      <c r="P31" s="34"/>
+      <c r="Q31" s="34"/>
+      <c r="R31" s="34"/>
+      <c r="S31" s="34"/>
+      <c r="T31" s="34"/>
+      <c r="U31" s="34"/>
+      <c r="V31" s="34"/>
+      <c r="W31" s="34"/>
+      <c r="X31" s="34"/>
+      <c r="Y31" s="34"/>
+      <c r="Z31" s="34"/>
+    </row>
+    <row r="32" ht="30.0" customHeight="1">
+      <c r="A32" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B32" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="C32" s="33" t="s">
+        <v>92</v>
+      </c>
+      <c r="D32" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="E32" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="F32" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="G32" s="33" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33" ht="30.0" customHeight="1">
+      <c r="A33" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B33" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>94</v>
+      </c>
+      <c r="D33" s="33" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="32">
         <v>2.0</v>
       </c>
-      <c r="F21" s="24">
+      <c r="F33" s="32">
         <v>2.0</v>
       </c>
-      <c r="G21" s="23" t="s">
+      <c r="G33" s="33" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="34" ht="30.0" customHeight="1">
+      <c r="A34" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="36" t="s">
+        <v>95</v>
+      </c>
+      <c r="C34" s="33" t="s">
+        <v>96</v>
+      </c>
+      <c r="D34" s="33" t="s">
+        <v>83</v>
+      </c>
+      <c r="E34" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="F34" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="G34" s="33" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="35" ht="30.0" customHeight="1">
+      <c r="A35" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="36" t="s">
+        <v>97</v>
+      </c>
+      <c r="C35" s="33" t="s">
+        <v>98</v>
+      </c>
+      <c r="D35" s="33" t="s">
+        <v>62</v>
+      </c>
+      <c r="E35" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="F35" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="G35" s="33" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="36" ht="30.0" customHeight="1">
+      <c r="A36" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" s="36" t="s">
+        <v>99</v>
+      </c>
+      <c r="C36" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="D36" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="E36" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="F36" s="32">
+        <v>1.0</v>
+      </c>
+      <c r="G36" s="33" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="37" ht="30.0" customHeight="1">
+      <c r="A37" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="B37" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="C37" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="D37" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="E37" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="F37" s="39">
+        <v>1.0</v>
+      </c>
+      <c r="G37" s="38" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="38" ht="30.0" customHeight="1">
+      <c r="A38" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B38" s="40" t="s">
+        <v>104</v>
+      </c>
+      <c r="C38" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="D38" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="E38" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="F38" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="G38" s="41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="39" ht="30.0" customHeight="1">
+      <c r="A39" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B39" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="C39" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="D39" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="E39" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="F39" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="G39" s="41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="40" ht="30.0" customHeight="1">
+      <c r="A40" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B40" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="C40" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="D40" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E40" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F40" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G40" s="41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="41" ht="30.0" customHeight="1">
+      <c r="A41" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B41" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="C41" s="41" t="s">
+        <v>111</v>
+      </c>
+      <c r="D41" s="41" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="22" ht="30.0" customHeight="1">
-      <c r="A22" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22" s="22" t="s">
+      <c r="E41" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="F41" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="G41" s="41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" ht="30.0" customHeight="1">
+      <c r="A42" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B42" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="C42" s="41" t="s">
+        <v>113</v>
+      </c>
+      <c r="D42" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="E42" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F42" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G42" s="41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="43" ht="30.0" customHeight="1">
+      <c r="A43" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B43" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="D43" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="23" t="s">
-        <v>63</v>
-      </c>
-      <c r="D22" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="E22" s="24">
+      <c r="E43" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="F43" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="G43" s="41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" ht="30.0" customHeight="1">
+      <c r="A44" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="B44" s="40" t="s">
+        <v>116</v>
+      </c>
+      <c r="C44" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="D44" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="E44" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="F44" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="G44" s="41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="45" ht="30.0" customHeight="1">
+      <c r="A45" s="43" t="s">
+        <v>103</v>
+      </c>
+      <c r="B45" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" s="44" t="s">
+        <v>119</v>
+      </c>
+      <c r="D45" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="E45" s="46">
+        <v>1.0</v>
+      </c>
+      <c r="F45" s="46">
+        <v>1.0</v>
+      </c>
+      <c r="G45" s="44" t="s">
+        <v>59</v>
+      </c>
+      <c r="H45" s="47"/>
+      <c r="I45" s="47"/>
+      <c r="J45" s="47"/>
+      <c r="K45" s="47"/>
+      <c r="L45" s="47"/>
+      <c r="M45" s="47"/>
+      <c r="N45" s="47"/>
+      <c r="O45" s="47"/>
+      <c r="P45" s="47"/>
+      <c r="Q45" s="47"/>
+      <c r="R45" s="47"/>
+      <c r="S45" s="47"/>
+      <c r="T45" s="47"/>
+      <c r="U45" s="47"/>
+      <c r="V45" s="47"/>
+      <c r="W45" s="47"/>
+      <c r="X45" s="47"/>
+      <c r="Y45" s="47"/>
+      <c r="Z45" s="47"/>
+    </row>
+    <row r="46" ht="30.0" customHeight="1">
+      <c r="A46" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="B46" s="40" t="s">
+        <v>121</v>
+      </c>
+      <c r="C46" s="41" t="s">
+        <v>122</v>
+      </c>
+      <c r="D46" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="E46" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F46" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G46" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="47" ht="30.0" customHeight="1">
+      <c r="A47" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="B47" s="40" t="s">
+        <v>123</v>
+      </c>
+      <c r="C47" s="41" t="s">
+        <v>124</v>
+      </c>
+      <c r="D47" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E47" s="42">
         <v>3.0</v>
       </c>
-      <c r="F22" s="24">
+      <c r="F47" s="42">
         <v>3.0</v>
       </c>
-      <c r="G22" s="23" t="s">
+      <c r="G47" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="48" ht="30.0" customHeight="1">
+      <c r="A48" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="B48" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" s="41" t="s">
+        <v>126</v>
+      </c>
+      <c r="D48" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="E48" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F48" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G48" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="49" ht="30.0" customHeight="1">
+      <c r="A49" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B49" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="C49" s="41" t="s">
+        <v>129</v>
+      </c>
+      <c r="D49" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="E49" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="F49" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="G49" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="50" ht="30.0" customHeight="1">
+      <c r="A50" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B50" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="C50" s="41" t="s">
+        <v>131</v>
+      </c>
+      <c r="D50" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E50" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F50" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G50" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="51" ht="30.0" customHeight="1">
+      <c r="A51" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B51" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="C51" s="41" t="s">
+        <v>133</v>
+      </c>
+      <c r="D51" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="E51" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="F51" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="G51" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="52" ht="30.0" customHeight="1">
+      <c r="A52" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="B52" s="40" t="s">
+        <v>135</v>
+      </c>
+      <c r="C52" s="41" t="s">
+        <v>136</v>
+      </c>
+      <c r="D52" s="41" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="23" ht="30.0" customHeight="1">
-      <c r="A23" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B23" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="C23" s="23" t="s">
-        <v>66</v>
-      </c>
-      <c r="D23" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="E23" s="24">
+      <c r="E52" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F52" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G52" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="53" ht="30.0" customHeight="1">
+      <c r="A53" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="B53" s="40" t="s">
+        <v>137</v>
+      </c>
+      <c r="C53" s="41" t="s">
+        <v>138</v>
+      </c>
+      <c r="D53" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="E53" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F53" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G53" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="54" ht="30.0" customHeight="1">
+      <c r="A54" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="B54" s="40" t="s">
+        <v>139</v>
+      </c>
+      <c r="C54" s="41" t="s">
+        <v>140</v>
+      </c>
+      <c r="D54" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="E54" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F54" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G54" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="55" ht="30.0" customHeight="1">
+      <c r="A55" s="40" t="s">
+        <v>141</v>
+      </c>
+      <c r="B55" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="C55" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="D55" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="E55" s="42">
         <v>1.0</v>
       </c>
-      <c r="F23" s="24">
+      <c r="F55" s="42">
         <v>1.0</v>
       </c>
-      <c r="G23" s="25" t="s">
+      <c r="G55" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="56" ht="30.0" customHeight="1">
+      <c r="A56" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="B56" s="40" t="s">
+        <v>145</v>
+      </c>
+      <c r="C56" s="41" t="s">
+        <v>146</v>
+      </c>
+      <c r="D56" s="41" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="24" ht="30.0" customHeight="1">
-      <c r="A24" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="B24" s="26" t="s">
+      <c r="E56" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F56" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G56" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="57" ht="30.0" customHeight="1">
+      <c r="A57" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="B57" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="C57" s="41" t="s">
+        <v>149</v>
+      </c>
+      <c r="D57" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="E57" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="F57" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="G57" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="58" ht="14.25" customHeight="1">
+      <c r="A58" s="48" t="s">
+        <v>150</v>
+      </c>
+      <c r="B58" s="49"/>
+      <c r="C58" s="50" t="s">
+        <v>151</v>
+      </c>
+      <c r="D58" s="49"/>
+      <c r="E58" s="51">
+        <v>36.0</v>
+      </c>
+      <c r="F58" s="51">
+        <v>34.0</v>
+      </c>
+      <c r="G58" s="49"/>
+    </row>
+    <row r="59" ht="14.25" customHeight="1"/>
+    <row r="60" ht="14.25" customHeight="1">
+      <c r="A60" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="61" ht="14.25" customHeight="1">
+      <c r="A61" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61" s="9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="62" ht="14.25" customHeight="1">
+      <c r="A62" s="53" t="s">
         <v>69</v>
       </c>
-      <c r="C24" s="23" t="s">
-        <v>70</v>
-      </c>
-      <c r="D24" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="E24" s="24">
-        <v>1.0</v>
-      </c>
-      <c r="F24" s="24">
-        <v>1.0</v>
-      </c>
-      <c r="G24" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
-      <c r="J24" s="27"/>
-      <c r="K24" s="27"/>
-      <c r="L24" s="27"/>
-      <c r="M24" s="27"/>
-      <c r="N24" s="27"/>
-      <c r="O24" s="27"/>
-      <c r="P24" s="27"/>
-      <c r="Q24" s="27"/>
-      <c r="R24" s="27"/>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
-      <c r="U24" s="27"/>
-      <c r="V24" s="27"/>
-      <c r="W24" s="27"/>
-      <c r="X24" s="27"/>
-      <c r="Y24" s="27"/>
-      <c r="Z24" s="27"/>
-    </row>
-    <row r="25" ht="30.0" customHeight="1">
-      <c r="A25" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="B25" s="28" t="s">
-        <v>72</v>
-      </c>
-      <c r="C25" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="D25" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="E25" s="30">
-        <v>1.0</v>
-      </c>
-      <c r="F25" s="30">
-        <v>1.0</v>
-      </c>
-      <c r="G25" s="29" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="26" ht="30.0" customHeight="1">
-      <c r="A26" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="B26" s="28" t="s">
-        <v>74</v>
-      </c>
-      <c r="C26" s="29" t="s">
-        <v>75</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>76</v>
-      </c>
-      <c r="E26" s="30">
-        <v>3.0</v>
-      </c>
-      <c r="F26" s="30">
-        <v>3.0</v>
-      </c>
-      <c r="G26" s="29" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="27" ht="30.0" customHeight="1">
-      <c r="A27" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="B27" s="28" t="s">
-        <v>77</v>
-      </c>
-      <c r="C27" s="29" t="s">
-        <v>78</v>
-      </c>
-      <c r="D27" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="E27" s="30">
-        <v>1.0</v>
-      </c>
-      <c r="F27" s="31">
-        <v>0.0</v>
-      </c>
-      <c r="G27" s="32" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="28" ht="30.0" customHeight="1">
-      <c r="A28" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="B28" s="28" t="s">
+      <c r="B62" s="9" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="63" ht="14.25" customHeight="1">
+      <c r="A63" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="B63" s="9" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="64" ht="14.25" customHeight="1">
+      <c r="A64" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="C28" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="D28" s="29" t="s">
-        <v>82</v>
-      </c>
-      <c r="E28" s="30">
-        <v>3.0</v>
-      </c>
-      <c r="F28" s="30">
-        <v>3.0</v>
-      </c>
-      <c r="G28" s="29" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" ht="30.0" customHeight="1">
-      <c r="A29" s="28" t="s">
-        <v>71</v>
-      </c>
-      <c r="B29" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="C29" s="29" t="s">
-        <v>84</v>
-      </c>
-      <c r="D29" s="29" t="s">
-        <v>67</v>
-      </c>
-      <c r="E29" s="30">
-        <v>1.0</v>
-      </c>
-      <c r="F29" s="31">
-        <v>0.0</v>
-      </c>
-      <c r="G29" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="H29" s="33"/>
-      <c r="I29" s="33"/>
-      <c r="J29" s="33"/>
-      <c r="K29" s="33"/>
-      <c r="L29" s="33"/>
-      <c r="M29" s="33"/>
-      <c r="N29" s="33"/>
-      <c r="O29" s="33"/>
-      <c r="P29" s="33"/>
-      <c r="Q29" s="33"/>
-      <c r="R29" s="33"/>
-      <c r="S29" s="33"/>
-      <c r="T29" s="33"/>
-      <c r="U29" s="33"/>
-      <c r="V29" s="33"/>
-      <c r="W29" s="33"/>
-      <c r="X29" s="33"/>
-      <c r="Y29" s="33"/>
-      <c r="Z29" s="33"/>
-    </row>
-    <row r="30" ht="30.0" customHeight="1">
-      <c r="A30" s="34" t="s">
-        <v>71</v>
-      </c>
-      <c r="B30" s="34" t="s">
-        <v>85</v>
-      </c>
-      <c r="C30" s="29" t="s">
-        <v>86</v>
-      </c>
-      <c r="D30" s="29" t="s">
-        <v>61</v>
-      </c>
-      <c r="E30" s="30">
-        <v>1.0</v>
-      </c>
-      <c r="F30" s="30">
-        <v>1.0</v>
-      </c>
-      <c r="G30" s="29" t="s">
-        <v>58</v>
-      </c>
-      <c r="H30" s="33"/>
-      <c r="I30" s="33"/>
-      <c r="J30" s="33"/>
-      <c r="K30" s="33"/>
-      <c r="L30" s="33"/>
-      <c r="M30" s="33"/>
-      <c r="N30" s="33"/>
-      <c r="O30" s="33"/>
-      <c r="P30" s="33"/>
-      <c r="Q30" s="33"/>
-      <c r="R30" s="33"/>
-      <c r="S30" s="33"/>
-      <c r="T30" s="33"/>
-      <c r="U30" s="33"/>
-      <c r="V30" s="33"/>
-      <c r="W30" s="33"/>
-      <c r="X30" s="33"/>
-      <c r="Y30" s="33"/>
-      <c r="Z30" s="33"/>
-    </row>
-    <row r="31" ht="30.0" customHeight="1">
-      <c r="A31" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B31" s="35" t="s">
-        <v>88</v>
-      </c>
-      <c r="C31" s="32" t="s">
-        <v>89</v>
-      </c>
-      <c r="D31" s="32" t="s">
-        <v>67</v>
-      </c>
-      <c r="E31" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="F31" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="G31" s="32" t="s">
-        <v>58</v>
-      </c>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
-      <c r="J31" s="33"/>
-      <c r="K31" s="33"/>
-      <c r="L31" s="33"/>
-      <c r="M31" s="33"/>
-      <c r="N31" s="33"/>
-      <c r="O31" s="33"/>
-      <c r="P31" s="33"/>
-      <c r="Q31" s="33"/>
-      <c r="R31" s="33"/>
-      <c r="S31" s="33"/>
-      <c r="T31" s="33"/>
-      <c r="U31" s="33"/>
-      <c r="V31" s="33"/>
-      <c r="W31" s="33"/>
-      <c r="X31" s="33"/>
-      <c r="Y31" s="33"/>
-      <c r="Z31" s="33"/>
-    </row>
-    <row r="32" ht="30.0" customHeight="1">
-      <c r="A32" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B32" s="35" t="s">
-        <v>90</v>
-      </c>
-      <c r="C32" s="32" t="s">
-        <v>91</v>
-      </c>
-      <c r="D32" s="32" t="s">
-        <v>57</v>
-      </c>
-      <c r="E32" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="F32" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="G32" s="32" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="33" ht="30.0" customHeight="1">
-      <c r="A33" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B33" s="35" t="s">
-        <v>92</v>
-      </c>
-      <c r="C33" s="32" t="s">
-        <v>93</v>
-      </c>
-      <c r="D33" s="32" t="s">
-        <v>76</v>
-      </c>
-      <c r="E33" s="31">
-        <v>2.0</v>
-      </c>
-      <c r="F33" s="31">
-        <v>2.0</v>
-      </c>
-      <c r="G33" s="32" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="34" ht="30.0" customHeight="1">
-      <c r="A34" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B34" s="35" t="s">
-        <v>94</v>
-      </c>
-      <c r="C34" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="D34" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="E34" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="F34" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="G34" s="32" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="35" ht="30.0" customHeight="1">
-      <c r="A35" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B35" s="35" t="s">
-        <v>96</v>
-      </c>
-      <c r="C35" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="D35" s="32" t="s">
-        <v>61</v>
-      </c>
-      <c r="E35" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="F35" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="G35" s="32" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="36" ht="30.0" customHeight="1">
-      <c r="A36" s="35" t="s">
-        <v>87</v>
-      </c>
-      <c r="B36" s="35" t="s">
-        <v>98</v>
-      </c>
-      <c r="C36" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="D36" s="32" t="s">
-        <v>64</v>
-      </c>
-      <c r="E36" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="F36" s="31">
-        <v>1.0</v>
-      </c>
-      <c r="G36" s="32" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="37" ht="30.0" customHeight="1">
-      <c r="A37" s="36" t="s">
-        <v>87</v>
-      </c>
-      <c r="B37" s="36" t="s">
-        <v>100</v>
-      </c>
-      <c r="C37" s="37" t="s">
-        <v>101</v>
-      </c>
-      <c r="D37" s="37" t="s">
-        <v>67</v>
-      </c>
-      <c r="E37" s="38">
-        <v>1.0</v>
-      </c>
-      <c r="F37" s="38">
-        <v>1.0</v>
-      </c>
-      <c r="G37" s="37" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="38" ht="30.0" customHeight="1">
-      <c r="A38" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B38" s="39" t="s">
-        <v>103</v>
-      </c>
-      <c r="C38" s="40" t="s">
-        <v>104</v>
-      </c>
-      <c r="D38" s="40"/>
-      <c r="E38" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="F38" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="G38" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="39" ht="30.0" customHeight="1">
-      <c r="A39" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B39" s="39" t="s">
-        <v>105</v>
-      </c>
-      <c r="C39" s="40" t="s">
-        <v>106</v>
-      </c>
-      <c r="D39" s="40"/>
-      <c r="E39" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="F39" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="G39" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="40" ht="30.0" customHeight="1">
-      <c r="A40" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B40" s="39" t="s">
-        <v>107</v>
-      </c>
-      <c r="C40" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="D40" s="40"/>
-      <c r="E40" s="41">
-        <v>2.0</v>
-      </c>
-      <c r="F40" s="41">
-        <v>2.0</v>
-      </c>
-      <c r="G40" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="41" ht="30.0" customHeight="1">
-      <c r="A41" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B41" s="39" t="s">
-        <v>109</v>
-      </c>
-      <c r="C41" s="40" t="s">
-        <v>110</v>
-      </c>
-      <c r="D41" s="40"/>
-      <c r="E41" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="F41" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="G41" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="42" ht="30.0" customHeight="1">
-      <c r="A42" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B42" s="39" t="s">
-        <v>111</v>
-      </c>
-      <c r="C42" s="40" t="s">
-        <v>112</v>
-      </c>
-      <c r="D42" s="40"/>
-      <c r="E42" s="41">
-        <v>2.0</v>
-      </c>
-      <c r="F42" s="41">
-        <v>2.0</v>
-      </c>
-      <c r="G42" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="43" ht="30.0" customHeight="1">
-      <c r="A43" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B43" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="C43" s="40" t="s">
-        <v>114</v>
-      </c>
-      <c r="D43" s="40"/>
-      <c r="E43" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="F43" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="G43" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="44" ht="30.0" customHeight="1">
-      <c r="A44" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B44" s="39" t="s">
-        <v>115</v>
-      </c>
-      <c r="C44" s="40" t="s">
-        <v>116</v>
-      </c>
-      <c r="D44" s="40"/>
-      <c r="E44" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="F44" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="G44" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="45" ht="30.0" customHeight="1">
-      <c r="A45" s="39" t="s">
-        <v>102</v>
-      </c>
-      <c r="B45" s="39" t="s">
-        <v>117</v>
-      </c>
-      <c r="C45" s="40" t="s">
-        <v>118</v>
-      </c>
-      <c r="D45" s="40"/>
-      <c r="E45" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="F45" s="41">
-        <v>1.0</v>
-      </c>
-      <c r="G45" s="40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="46" ht="14.25" customHeight="1">
-      <c r="A46" s="42" t="s">
-        <v>119</v>
-      </c>
-      <c r="B46" s="43"/>
-      <c r="C46" s="44" t="s">
-        <v>120</v>
-      </c>
-      <c r="D46" s="43"/>
-      <c r="E46" s="45">
-        <v>36.0</v>
-      </c>
-      <c r="F46" s="45">
-        <v>34.0</v>
-      </c>
-      <c r="G46" s="43"/>
-    </row>
-    <row r="47" ht="14.25" customHeight="1"/>
-    <row r="48" ht="14.25" customHeight="1">
-      <c r="A48" s="3" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="49" ht="14.25" customHeight="1">
-      <c r="A49" s="46" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49" s="9" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="50" ht="14.25" customHeight="1">
-      <c r="A50" s="47" t="s">
-        <v>68</v>
-      </c>
-      <c r="B50" s="9" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="51" ht="14.25" customHeight="1">
-      <c r="A51" s="20" t="s">
-        <v>124</v>
-      </c>
-      <c r="B51" s="9" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="52" ht="14.25" customHeight="1">
-      <c r="A52" s="19" t="s">
-        <v>79</v>
-      </c>
-      <c r="B52" s="9" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="53" ht="14.25" customHeight="1"/>
-    <row r="54" ht="14.25" customHeight="1"/>
-    <row r="55" ht="14.25" customHeight="1"/>
-    <row r="56" ht="14.25" customHeight="1"/>
-    <row r="57" ht="14.25" customHeight="1"/>
-    <row r="58" ht="14.25" customHeight="1"/>
-    <row r="59" ht="14.25" customHeight="1"/>
-    <row r="60" ht="14.25" customHeight="1"/>
-    <row r="61" ht="14.25" customHeight="1"/>
-    <row r="62" ht="14.25" customHeight="1"/>
-    <row r="63" ht="14.25" customHeight="1"/>
-    <row r="64" ht="14.25" customHeight="1"/>
+      <c r="B64" s="9" t="s">
+        <v>157</v>
+      </c>
+    </row>
     <row r="65" ht="14.25" customHeight="1"/>
     <row r="66" ht="14.25" customHeight="1"/>
     <row r="67" ht="14.25" customHeight="1"/>
@@ -5183,6 +5625,18 @@
     <row r="1014" ht="14.25" customHeight="1"/>
     <row r="1015" ht="14.25" customHeight="1"/>
     <row r="1016" ht="14.25" customHeight="1"/>
+    <row r="1017" ht="14.25" customHeight="1"/>
+    <row r="1018" ht="14.25" customHeight="1"/>
+    <row r="1019" ht="14.25" customHeight="1"/>
+    <row r="1020" ht="14.25" customHeight="1"/>
+    <row r="1021" ht="14.25" customHeight="1"/>
+    <row r="1022" ht="14.25" customHeight="1"/>
+    <row r="1023" ht="14.25" customHeight="1"/>
+    <row r="1024" ht="14.25" customHeight="1"/>
+    <row r="1025" ht="14.25" customHeight="1"/>
+    <row r="1026" ht="14.25" customHeight="1"/>
+    <row r="1027" ht="14.25" customHeight="1"/>
+    <row r="1028" ht="14.25" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -5198,6 +5652,1462 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
+    <col customWidth="1" min="1" max="1" width="15.71"/>
+    <col customWidth="1" min="2" max="2" width="22.86"/>
+    <col customWidth="1" min="3" max="3" width="89.29"/>
+    <col customWidth="1" min="4" max="4" width="13.0"/>
+    <col customWidth="1" min="5" max="5" width="10.0"/>
+    <col customWidth="1" min="6" max="7" width="11.0"/>
+    <col customWidth="1" min="8" max="26" width="8.86"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="44.25" customHeight="1">
+      <c r="A1" s="15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" ht="14.25" customHeight="1">
+      <c r="A2" s="16" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3" ht="14.25" customHeight="1"/>
+    <row r="4" ht="14.25" customHeight="1">
+      <c r="A4" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" ht="21.75" customHeight="1">
+      <c r="A5" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" ht="27.75" customHeight="1">
+      <c r="A6" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7" ht="21.75" customHeight="1">
+      <c r="A7" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" ht="21.75" customHeight="1">
+      <c r="A8" s="17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" ht="30.0" customHeight="1">
+      <c r="A9" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="10" ht="81.0" customHeight="1">
+      <c r="A10" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" ht="21.75" customHeight="1">
+      <c r="A11" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" ht="21.75" customHeight="1">
+      <c r="A12" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" ht="14.25" customHeight="1"/>
+    <row r="14" ht="14.25" customHeight="1">
+      <c r="A14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25" customHeight="1">
+      <c r="A15" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25" customHeight="1">
+      <c r="A16" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25" customHeight="1">
+      <c r="A17" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25" customHeight="1"/>
+    <row r="19" ht="14.25" customHeight="1">
+      <c r="A19" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="22" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" ht="30.0" customHeight="1">
+      <c r="A20" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" s="40" t="s">
+        <v>121</v>
+      </c>
+      <c r="C20" s="41" t="s">
+        <v>122</v>
+      </c>
+      <c r="D20" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="E20" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F20" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G20" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" ht="30.0" customHeight="1">
+      <c r="A21" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" s="40" t="s">
+        <v>123</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>124</v>
+      </c>
+      <c r="D21" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E21" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="F21" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="G21" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" ht="30.0" customHeight="1">
+      <c r="A22" s="40" t="s">
+        <v>120</v>
+      </c>
+      <c r="B22" s="40" t="s">
+        <v>125</v>
+      </c>
+      <c r="C22" s="41" t="s">
+        <v>126</v>
+      </c>
+      <c r="D22" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="E22" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F22" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G22" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" ht="30.0" customHeight="1">
+      <c r="A23" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B23" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="C23" s="41" t="s">
+        <v>129</v>
+      </c>
+      <c r="D23" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="E23" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="F23" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="G23" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" ht="30.0" customHeight="1">
+      <c r="A24" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B24" s="40" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="41" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" s="41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F24" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G24" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" ht="30.0" customHeight="1">
+      <c r="A25" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="B25" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="C25" s="41" t="s">
+        <v>133</v>
+      </c>
+      <c r="D25" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="F25" s="42">
+        <v>3.0</v>
+      </c>
+      <c r="G25" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="26" ht="30.0" customHeight="1">
+      <c r="A26" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" s="40" t="s">
+        <v>135</v>
+      </c>
+      <c r="C26" s="41" t="s">
+        <v>136</v>
+      </c>
+      <c r="D26" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F26" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G26" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" ht="30.0" customHeight="1">
+      <c r="A27" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="B27" s="40" t="s">
+        <v>137</v>
+      </c>
+      <c r="C27" s="41" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="E27" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F27" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G27" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="28" ht="30.0" customHeight="1">
+      <c r="A28" s="40" t="s">
+        <v>134</v>
+      </c>
+      <c r="B28" s="40" t="s">
+        <v>139</v>
+      </c>
+      <c r="C28" s="41" t="s">
+        <v>140</v>
+      </c>
+      <c r="D28" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="E28" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F28" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G28" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" ht="30.0" customHeight="1">
+      <c r="A29" s="40" t="s">
+        <v>141</v>
+      </c>
+      <c r="B29" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="C29" s="41" t="s">
+        <v>143</v>
+      </c>
+      <c r="D29" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="E29" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="F29" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="G29" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" ht="30.0" customHeight="1">
+      <c r="A30" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="B30" s="40" t="s">
+        <v>145</v>
+      </c>
+      <c r="C30" s="41" t="s">
+        <v>146</v>
+      </c>
+      <c r="D30" s="41" t="s">
+        <v>68</v>
+      </c>
+      <c r="E30" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="F30" s="42">
+        <v>2.0</v>
+      </c>
+      <c r="G30" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="31" ht="30.0" customHeight="1">
+      <c r="A31" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="B31" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="C31" s="41" t="s">
+        <v>149</v>
+      </c>
+      <c r="D31" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="F31" s="42">
+        <v>1.0</v>
+      </c>
+      <c r="G31" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="32" ht="14.25" customHeight="1">
+      <c r="A32" s="48" t="s">
+        <v>150</v>
+      </c>
+      <c r="B32" s="49"/>
+      <c r="C32" s="50" t="s">
+        <v>162</v>
+      </c>
+      <c r="D32" s="49"/>
+      <c r="E32" s="51">
+        <v>25.0</v>
+      </c>
+      <c r="F32" s="51">
+        <v>25.0</v>
+      </c>
+      <c r="G32" s="49"/>
+    </row>
+    <row r="33" ht="14.25" customHeight="1"/>
+    <row r="34" ht="14.25" customHeight="1">
+      <c r="A34" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="35" ht="14.25" customHeight="1">
+      <c r="A35" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" ht="14.25" customHeight="1">
+      <c r="A36" s="53" t="s">
+        <v>69</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="37" ht="14.25" customHeight="1">
+      <c r="A37" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="B37" s="9" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="38" ht="14.25" customHeight="1">
+      <c r="A38" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" s="9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="39" ht="14.25" customHeight="1"/>
+    <row r="40" ht="14.25" customHeight="1"/>
+    <row r="41" ht="14.25" customHeight="1"/>
+    <row r="42" ht="14.25" customHeight="1"/>
+    <row r="43" ht="14.25" customHeight="1"/>
+    <row r="44" ht="14.25" customHeight="1"/>
+    <row r="45" ht="14.25" customHeight="1"/>
+    <row r="46" ht="14.25" customHeight="1"/>
+    <row r="47" ht="14.25" customHeight="1"/>
+    <row r="48" ht="14.25" customHeight="1"/>
+    <row r="49" ht="14.25" customHeight="1"/>
+    <row r="50" ht="14.25" customHeight="1"/>
+    <row r="51" ht="14.25" customHeight="1"/>
+    <row r="52" ht="14.25" customHeight="1"/>
+    <row r="53" ht="14.25" customHeight="1"/>
+    <row r="54" ht="14.25" customHeight="1"/>
+    <row r="55" ht="14.25" customHeight="1"/>
+    <row r="56" ht="14.25" customHeight="1"/>
+    <row r="57" ht="14.25" customHeight="1"/>
+    <row r="58" ht="14.25" customHeight="1"/>
+    <row r="59" ht="14.25" customHeight="1"/>
+    <row r="60" ht="14.25" customHeight="1"/>
+    <row r="61" ht="14.25" customHeight="1"/>
+    <row r="62" ht="14.25" customHeight="1"/>
+    <row r="63" ht="14.25" customHeight="1"/>
+    <row r="64" ht="14.25" customHeight="1"/>
+    <row r="65" ht="14.25" customHeight="1"/>
+    <row r="66" ht="14.25" customHeight="1"/>
+    <row r="67" ht="14.25" customHeight="1"/>
+    <row r="68" ht="14.25" customHeight="1"/>
+    <row r="69" ht="14.25" customHeight="1"/>
+    <row r="70" ht="14.25" customHeight="1"/>
+    <row r="71" ht="14.25" customHeight="1"/>
+    <row r="72" ht="14.25" customHeight="1"/>
+    <row r="73" ht="14.25" customHeight="1"/>
+    <row r="74" ht="14.25" customHeight="1"/>
+    <row r="75" ht="14.25" customHeight="1"/>
+    <row r="76" ht="14.25" customHeight="1"/>
+    <row r="77" ht="14.25" customHeight="1"/>
+    <row r="78" ht="14.25" customHeight="1"/>
+    <row r="79" ht="14.25" customHeight="1"/>
+    <row r="80" ht="14.25" customHeight="1"/>
+    <row r="81" ht="14.25" customHeight="1"/>
+    <row r="82" ht="14.25" customHeight="1"/>
+    <row r="83" ht="14.25" customHeight="1"/>
+    <row r="84" ht="14.25" customHeight="1"/>
+    <row r="85" ht="14.25" customHeight="1"/>
+    <row r="86" ht="14.25" customHeight="1"/>
+    <row r="87" ht="14.25" customHeight="1"/>
+    <row r="88" ht="14.25" customHeight="1"/>
+    <row r="89" ht="14.25" customHeight="1"/>
+    <row r="90" ht="14.25" customHeight="1"/>
+    <row r="91" ht="14.25" customHeight="1"/>
+    <row r="92" ht="14.25" customHeight="1"/>
+    <row r="93" ht="14.25" customHeight="1"/>
+    <row r="94" ht="14.25" customHeight="1"/>
+    <row r="95" ht="14.25" customHeight="1"/>
+    <row r="96" ht="14.25" customHeight="1"/>
+    <row r="97" ht="14.25" customHeight="1"/>
+    <row r="98" ht="14.25" customHeight="1"/>
+    <row r="99" ht="14.25" customHeight="1"/>
+    <row r="100" ht="14.25" customHeight="1"/>
+    <row r="101" ht="14.25" customHeight="1"/>
+    <row r="102" ht="14.25" customHeight="1"/>
+    <row r="103" ht="14.25" customHeight="1"/>
+    <row r="104" ht="14.25" customHeight="1"/>
+    <row r="105" ht="14.25" customHeight="1"/>
+    <row r="106" ht="14.25" customHeight="1"/>
+    <row r="107" ht="14.25" customHeight="1"/>
+    <row r="108" ht="14.25" customHeight="1"/>
+    <row r="109" ht="14.25" customHeight="1"/>
+    <row r="110" ht="14.25" customHeight="1"/>
+    <row r="111" ht="14.25" customHeight="1"/>
+    <row r="112" ht="14.25" customHeight="1"/>
+    <row r="113" ht="14.25" customHeight="1"/>
+    <row r="114" ht="14.25" customHeight="1"/>
+    <row r="115" ht="14.25" customHeight="1"/>
+    <row r="116" ht="14.25" customHeight="1"/>
+    <row r="117" ht="14.25" customHeight="1"/>
+    <row r="118" ht="14.25" customHeight="1"/>
+    <row r="119" ht="14.25" customHeight="1"/>
+    <row r="120" ht="14.25" customHeight="1"/>
+    <row r="121" ht="14.25" customHeight="1"/>
+    <row r="122" ht="14.25" customHeight="1"/>
+    <row r="123" ht="14.25" customHeight="1"/>
+    <row r="124" ht="14.25" customHeight="1"/>
+    <row r="125" ht="14.25" customHeight="1"/>
+    <row r="126" ht="14.25" customHeight="1"/>
+    <row r="127" ht="14.25" customHeight="1"/>
+    <row r="128" ht="14.25" customHeight="1"/>
+    <row r="129" ht="14.25" customHeight="1"/>
+    <row r="130" ht="14.25" customHeight="1"/>
+    <row r="131" ht="14.25" customHeight="1"/>
+    <row r="132" ht="14.25" customHeight="1"/>
+    <row r="133" ht="14.25" customHeight="1"/>
+    <row r="134" ht="14.25" customHeight="1"/>
+    <row r="135" ht="14.25" customHeight="1"/>
+    <row r="136" ht="14.25" customHeight="1"/>
+    <row r="137" ht="14.25" customHeight="1"/>
+    <row r="138" ht="14.25" customHeight="1"/>
+    <row r="139" ht="14.25" customHeight="1"/>
+    <row r="140" ht="14.25" customHeight="1"/>
+    <row r="141" ht="14.25" customHeight="1"/>
+    <row r="142" ht="14.25" customHeight="1"/>
+    <row r="143" ht="14.25" customHeight="1"/>
+    <row r="144" ht="14.25" customHeight="1"/>
+    <row r="145" ht="14.25" customHeight="1"/>
+    <row r="146" ht="14.25" customHeight="1"/>
+    <row r="147" ht="14.25" customHeight="1"/>
+    <row r="148" ht="14.25" customHeight="1"/>
+    <row r="149" ht="14.25" customHeight="1"/>
+    <row r="150" ht="14.25" customHeight="1"/>
+    <row r="151" ht="14.25" customHeight="1"/>
+    <row r="152" ht="14.25" customHeight="1"/>
+    <row r="153" ht="14.25" customHeight="1"/>
+    <row r="154" ht="14.25" customHeight="1"/>
+    <row r="155" ht="14.25" customHeight="1"/>
+    <row r="156" ht="14.25" customHeight="1"/>
+    <row r="157" ht="14.25" customHeight="1"/>
+    <row r="158" ht="14.25" customHeight="1"/>
+    <row r="159" ht="14.25" customHeight="1"/>
+    <row r="160" ht="14.25" customHeight="1"/>
+    <row r="161" ht="14.25" customHeight="1"/>
+    <row r="162" ht="14.25" customHeight="1"/>
+    <row r="163" ht="14.25" customHeight="1"/>
+    <row r="164" ht="14.25" customHeight="1"/>
+    <row r="165" ht="14.25" customHeight="1"/>
+    <row r="166" ht="14.25" customHeight="1"/>
+    <row r="167" ht="14.25" customHeight="1"/>
+    <row r="168" ht="14.25" customHeight="1"/>
+    <row r="169" ht="14.25" customHeight="1"/>
+    <row r="170" ht="14.25" customHeight="1"/>
+    <row r="171" ht="14.25" customHeight="1"/>
+    <row r="172" ht="14.25" customHeight="1"/>
+    <row r="173" ht="14.25" customHeight="1"/>
+    <row r="174" ht="14.25" customHeight="1"/>
+    <row r="175" ht="14.25" customHeight="1"/>
+    <row r="176" ht="14.25" customHeight="1"/>
+    <row r="177" ht="14.25" customHeight="1"/>
+    <row r="178" ht="14.25" customHeight="1"/>
+    <row r="179" ht="14.25" customHeight="1"/>
+    <row r="180" ht="14.25" customHeight="1"/>
+    <row r="181" ht="14.25" customHeight="1"/>
+    <row r="182" ht="14.25" customHeight="1"/>
+    <row r="183" ht="14.25" customHeight="1"/>
+    <row r="184" ht="14.25" customHeight="1"/>
+    <row r="185" ht="14.25" customHeight="1"/>
+    <row r="186" ht="14.25" customHeight="1"/>
+    <row r="187" ht="14.25" customHeight="1"/>
+    <row r="188" ht="14.25" customHeight="1"/>
+    <row r="189" ht="14.25" customHeight="1"/>
+    <row r="190" ht="14.25" customHeight="1"/>
+    <row r="191" ht="14.25" customHeight="1"/>
+    <row r="192" ht="14.25" customHeight="1"/>
+    <row r="193" ht="14.25" customHeight="1"/>
+    <row r="194" ht="14.25" customHeight="1"/>
+    <row r="195" ht="14.25" customHeight="1"/>
+    <row r="196" ht="14.25" customHeight="1"/>
+    <row r="197" ht="14.25" customHeight="1"/>
+    <row r="198" ht="14.25" customHeight="1"/>
+    <row r="199" ht="14.25" customHeight="1"/>
+    <row r="200" ht="14.25" customHeight="1"/>
+    <row r="201" ht="14.25" customHeight="1"/>
+    <row r="202" ht="14.25" customHeight="1"/>
+    <row r="203" ht="14.25" customHeight="1"/>
+    <row r="204" ht="14.25" customHeight="1"/>
+    <row r="205" ht="14.25" customHeight="1"/>
+    <row r="206" ht="14.25" customHeight="1"/>
+    <row r="207" ht="14.25" customHeight="1"/>
+    <row r="208" ht="14.25" customHeight="1"/>
+    <row r="209" ht="14.25" customHeight="1"/>
+    <row r="210" ht="14.25" customHeight="1"/>
+    <row r="211" ht="14.25" customHeight="1"/>
+    <row r="212" ht="14.25" customHeight="1"/>
+    <row r="213" ht="14.25" customHeight="1"/>
+    <row r="214" ht="14.25" customHeight="1"/>
+    <row r="215" ht="14.25" customHeight="1"/>
+    <row r="216" ht="14.25" customHeight="1"/>
+    <row r="217" ht="14.25" customHeight="1"/>
+    <row r="218" ht="14.25" customHeight="1"/>
+    <row r="219" ht="14.25" customHeight="1"/>
+    <row r="220" ht="14.25" customHeight="1"/>
+    <row r="221" ht="14.25" customHeight="1"/>
+    <row r="222" ht="14.25" customHeight="1"/>
+    <row r="223" ht="14.25" customHeight="1"/>
+    <row r="224" ht="14.25" customHeight="1"/>
+    <row r="225" ht="14.25" customHeight="1"/>
+    <row r="226" ht="14.25" customHeight="1"/>
+    <row r="227" ht="14.25" customHeight="1"/>
+    <row r="228" ht="14.25" customHeight="1"/>
+    <row r="229" ht="14.25" customHeight="1"/>
+    <row r="230" ht="14.25" customHeight="1"/>
+    <row r="231" ht="14.25" customHeight="1"/>
+    <row r="232" ht="14.25" customHeight="1"/>
+    <row r="233" ht="14.25" customHeight="1"/>
+    <row r="234" ht="14.25" customHeight="1"/>
+    <row r="235" ht="14.25" customHeight="1"/>
+    <row r="236" ht="14.25" customHeight="1"/>
+    <row r="237" ht="14.25" customHeight="1"/>
+    <row r="238" ht="14.25" customHeight="1"/>
+    <row r="239" ht="14.25" customHeight="1"/>
+    <row r="240" ht="14.25" customHeight="1"/>
+    <row r="241" ht="14.25" customHeight="1"/>
+    <row r="242" ht="14.25" customHeight="1"/>
+    <row r="243" ht="14.25" customHeight="1"/>
+    <row r="244" ht="14.25" customHeight="1"/>
+    <row r="245" ht="14.25" customHeight="1"/>
+    <row r="246" ht="14.25" customHeight="1"/>
+    <row r="247" ht="14.25" customHeight="1"/>
+    <row r="248" ht="14.25" customHeight="1"/>
+    <row r="249" ht="14.25" customHeight="1"/>
+    <row r="250" ht="14.25" customHeight="1"/>
+    <row r="251" ht="14.25" customHeight="1"/>
+    <row r="252" ht="14.25" customHeight="1"/>
+    <row r="253" ht="14.25" customHeight="1"/>
+    <row r="254" ht="14.25" customHeight="1"/>
+    <row r="255" ht="14.25" customHeight="1"/>
+    <row r="256" ht="14.25" customHeight="1"/>
+    <row r="257" ht="14.25" customHeight="1"/>
+    <row r="258" ht="14.25" customHeight="1"/>
+    <row r="259" ht="14.25" customHeight="1"/>
+    <row r="260" ht="14.25" customHeight="1"/>
+    <row r="261" ht="14.25" customHeight="1"/>
+    <row r="262" ht="14.25" customHeight="1"/>
+    <row r="263" ht="14.25" customHeight="1"/>
+    <row r="264" ht="14.25" customHeight="1"/>
+    <row r="265" ht="14.25" customHeight="1"/>
+    <row r="266" ht="14.25" customHeight="1"/>
+    <row r="267" ht="14.25" customHeight="1"/>
+    <row r="268" ht="14.25" customHeight="1"/>
+    <row r="269" ht="14.25" customHeight="1"/>
+    <row r="270" ht="14.25" customHeight="1"/>
+    <row r="271" ht="14.25" customHeight="1"/>
+    <row r="272" ht="14.25" customHeight="1"/>
+    <row r="273" ht="14.25" customHeight="1"/>
+    <row r="274" ht="14.25" customHeight="1"/>
+    <row r="275" ht="14.25" customHeight="1"/>
+    <row r="276" ht="14.25" customHeight="1"/>
+    <row r="277" ht="14.25" customHeight="1"/>
+    <row r="278" ht="14.25" customHeight="1"/>
+    <row r="279" ht="14.25" customHeight="1"/>
+    <row r="280" ht="14.25" customHeight="1"/>
+    <row r="281" ht="14.25" customHeight="1"/>
+    <row r="282" ht="14.25" customHeight="1"/>
+    <row r="283" ht="14.25" customHeight="1"/>
+    <row r="284" ht="14.25" customHeight="1"/>
+    <row r="285" ht="14.25" customHeight="1"/>
+    <row r="286" ht="14.25" customHeight="1"/>
+    <row r="287" ht="14.25" customHeight="1"/>
+    <row r="288" ht="14.25" customHeight="1"/>
+    <row r="289" ht="14.25" customHeight="1"/>
+    <row r="290" ht="14.25" customHeight="1"/>
+    <row r="291" ht="14.25" customHeight="1"/>
+    <row r="292" ht="14.25" customHeight="1"/>
+    <row r="293" ht="14.25" customHeight="1"/>
+    <row r="294" ht="14.25" customHeight="1"/>
+    <row r="295" ht="14.25" customHeight="1"/>
+    <row r="296" ht="14.25" customHeight="1"/>
+    <row r="297" ht="14.25" customHeight="1"/>
+    <row r="298" ht="14.25" customHeight="1"/>
+    <row r="299" ht="14.25" customHeight="1"/>
+    <row r="300" ht="14.25" customHeight="1"/>
+    <row r="301" ht="14.25" customHeight="1"/>
+    <row r="302" ht="14.25" customHeight="1"/>
+    <row r="303" ht="14.25" customHeight="1"/>
+    <row r="304" ht="14.25" customHeight="1"/>
+    <row r="305" ht="14.25" customHeight="1"/>
+    <row r="306" ht="14.25" customHeight="1"/>
+    <row r="307" ht="14.25" customHeight="1"/>
+    <row r="308" ht="14.25" customHeight="1"/>
+    <row r="309" ht="14.25" customHeight="1"/>
+    <row r="310" ht="14.25" customHeight="1"/>
+    <row r="311" ht="14.25" customHeight="1"/>
+    <row r="312" ht="14.25" customHeight="1"/>
+    <row r="313" ht="14.25" customHeight="1"/>
+    <row r="314" ht="14.25" customHeight="1"/>
+    <row r="315" ht="14.25" customHeight="1"/>
+    <row r="316" ht="14.25" customHeight="1"/>
+    <row r="317" ht="14.25" customHeight="1"/>
+    <row r="318" ht="14.25" customHeight="1"/>
+    <row r="319" ht="14.25" customHeight="1"/>
+    <row r="320" ht="14.25" customHeight="1"/>
+    <row r="321" ht="14.25" customHeight="1"/>
+    <row r="322" ht="14.25" customHeight="1"/>
+    <row r="323" ht="14.25" customHeight="1"/>
+    <row r="324" ht="14.25" customHeight="1"/>
+    <row r="325" ht="14.25" customHeight="1"/>
+    <row r="326" ht="14.25" customHeight="1"/>
+    <row r="327" ht="14.25" customHeight="1"/>
+    <row r="328" ht="14.25" customHeight="1"/>
+    <row r="329" ht="14.25" customHeight="1"/>
+    <row r="330" ht="14.25" customHeight="1"/>
+    <row r="331" ht="14.25" customHeight="1"/>
+    <row r="332" ht="14.25" customHeight="1"/>
+    <row r="333" ht="14.25" customHeight="1"/>
+    <row r="334" ht="14.25" customHeight="1"/>
+    <row r="335" ht="14.25" customHeight="1"/>
+    <row r="336" ht="14.25" customHeight="1"/>
+    <row r="337" ht="14.25" customHeight="1"/>
+    <row r="338" ht="14.25" customHeight="1"/>
+    <row r="339" ht="14.25" customHeight="1"/>
+    <row r="340" ht="14.25" customHeight="1"/>
+    <row r="341" ht="14.25" customHeight="1"/>
+    <row r="342" ht="14.25" customHeight="1"/>
+    <row r="343" ht="14.25" customHeight="1"/>
+    <row r="344" ht="14.25" customHeight="1"/>
+    <row r="345" ht="14.25" customHeight="1"/>
+    <row r="346" ht="14.25" customHeight="1"/>
+    <row r="347" ht="14.25" customHeight="1"/>
+    <row r="348" ht="14.25" customHeight="1"/>
+    <row r="349" ht="14.25" customHeight="1"/>
+    <row r="350" ht="14.25" customHeight="1"/>
+    <row r="351" ht="14.25" customHeight="1"/>
+    <row r="352" ht="14.25" customHeight="1"/>
+    <row r="353" ht="14.25" customHeight="1"/>
+    <row r="354" ht="14.25" customHeight="1"/>
+    <row r="355" ht="14.25" customHeight="1"/>
+    <row r="356" ht="14.25" customHeight="1"/>
+    <row r="357" ht="14.25" customHeight="1"/>
+    <row r="358" ht="14.25" customHeight="1"/>
+    <row r="359" ht="14.25" customHeight="1"/>
+    <row r="360" ht="14.25" customHeight="1"/>
+    <row r="361" ht="14.25" customHeight="1"/>
+    <row r="362" ht="14.25" customHeight="1"/>
+    <row r="363" ht="14.25" customHeight="1"/>
+    <row r="364" ht="14.25" customHeight="1"/>
+    <row r="365" ht="14.25" customHeight="1"/>
+    <row r="366" ht="14.25" customHeight="1"/>
+    <row r="367" ht="14.25" customHeight="1"/>
+    <row r="368" ht="14.25" customHeight="1"/>
+    <row r="369" ht="14.25" customHeight="1"/>
+    <row r="370" ht="14.25" customHeight="1"/>
+    <row r="371" ht="14.25" customHeight="1"/>
+    <row r="372" ht="14.25" customHeight="1"/>
+    <row r="373" ht="14.25" customHeight="1"/>
+    <row r="374" ht="14.25" customHeight="1"/>
+    <row r="375" ht="14.25" customHeight="1"/>
+    <row r="376" ht="14.25" customHeight="1"/>
+    <row r="377" ht="14.25" customHeight="1"/>
+    <row r="378" ht="14.25" customHeight="1"/>
+    <row r="379" ht="14.25" customHeight="1"/>
+    <row r="380" ht="14.25" customHeight="1"/>
+    <row r="381" ht="14.25" customHeight="1"/>
+    <row r="382" ht="14.25" customHeight="1"/>
+    <row r="383" ht="14.25" customHeight="1"/>
+    <row r="384" ht="14.25" customHeight="1"/>
+    <row r="385" ht="14.25" customHeight="1"/>
+    <row r="386" ht="14.25" customHeight="1"/>
+    <row r="387" ht="14.25" customHeight="1"/>
+    <row r="388" ht="14.25" customHeight="1"/>
+    <row r="389" ht="14.25" customHeight="1"/>
+    <row r="390" ht="14.25" customHeight="1"/>
+    <row r="391" ht="14.25" customHeight="1"/>
+    <row r="392" ht="14.25" customHeight="1"/>
+    <row r="393" ht="14.25" customHeight="1"/>
+    <row r="394" ht="14.25" customHeight="1"/>
+    <row r="395" ht="14.25" customHeight="1"/>
+    <row r="396" ht="14.25" customHeight="1"/>
+    <row r="397" ht="14.25" customHeight="1"/>
+    <row r="398" ht="14.25" customHeight="1"/>
+    <row r="399" ht="14.25" customHeight="1"/>
+    <row r="400" ht="14.25" customHeight="1"/>
+    <row r="401" ht="14.25" customHeight="1"/>
+    <row r="402" ht="14.25" customHeight="1"/>
+    <row r="403" ht="14.25" customHeight="1"/>
+    <row r="404" ht="14.25" customHeight="1"/>
+    <row r="405" ht="14.25" customHeight="1"/>
+    <row r="406" ht="14.25" customHeight="1"/>
+    <row r="407" ht="14.25" customHeight="1"/>
+    <row r="408" ht="14.25" customHeight="1"/>
+    <row r="409" ht="14.25" customHeight="1"/>
+    <row r="410" ht="14.25" customHeight="1"/>
+    <row r="411" ht="14.25" customHeight="1"/>
+    <row r="412" ht="14.25" customHeight="1"/>
+    <row r="413" ht="14.25" customHeight="1"/>
+    <row r="414" ht="14.25" customHeight="1"/>
+    <row r="415" ht="14.25" customHeight="1"/>
+    <row r="416" ht="14.25" customHeight="1"/>
+    <row r="417" ht="14.25" customHeight="1"/>
+    <row r="418" ht="14.25" customHeight="1"/>
+    <row r="419" ht="14.25" customHeight="1"/>
+    <row r="420" ht="14.25" customHeight="1"/>
+    <row r="421" ht="14.25" customHeight="1"/>
+    <row r="422" ht="14.25" customHeight="1"/>
+    <row r="423" ht="14.25" customHeight="1"/>
+    <row r="424" ht="14.25" customHeight="1"/>
+    <row r="425" ht="14.25" customHeight="1"/>
+    <row r="426" ht="14.25" customHeight="1"/>
+    <row r="427" ht="14.25" customHeight="1"/>
+    <row r="428" ht="14.25" customHeight="1"/>
+    <row r="429" ht="14.25" customHeight="1"/>
+    <row r="430" ht="14.25" customHeight="1"/>
+    <row r="431" ht="14.25" customHeight="1"/>
+    <row r="432" ht="14.25" customHeight="1"/>
+    <row r="433" ht="14.25" customHeight="1"/>
+    <row r="434" ht="14.25" customHeight="1"/>
+    <row r="435" ht="14.25" customHeight="1"/>
+    <row r="436" ht="14.25" customHeight="1"/>
+    <row r="437" ht="14.25" customHeight="1"/>
+    <row r="438" ht="14.25" customHeight="1"/>
+    <row r="439" ht="14.25" customHeight="1"/>
+    <row r="440" ht="14.25" customHeight="1"/>
+    <row r="441" ht="14.25" customHeight="1"/>
+    <row r="442" ht="14.25" customHeight="1"/>
+    <row r="443" ht="14.25" customHeight="1"/>
+    <row r="444" ht="14.25" customHeight="1"/>
+    <row r="445" ht="14.25" customHeight="1"/>
+    <row r="446" ht="14.25" customHeight="1"/>
+    <row r="447" ht="14.25" customHeight="1"/>
+    <row r="448" ht="14.25" customHeight="1"/>
+    <row r="449" ht="14.25" customHeight="1"/>
+    <row r="450" ht="14.25" customHeight="1"/>
+    <row r="451" ht="14.25" customHeight="1"/>
+    <row r="452" ht="14.25" customHeight="1"/>
+    <row r="453" ht="14.25" customHeight="1"/>
+    <row r="454" ht="14.25" customHeight="1"/>
+    <row r="455" ht="14.25" customHeight="1"/>
+    <row r="456" ht="14.25" customHeight="1"/>
+    <row r="457" ht="14.25" customHeight="1"/>
+    <row r="458" ht="14.25" customHeight="1"/>
+    <row r="459" ht="14.25" customHeight="1"/>
+    <row r="460" ht="14.25" customHeight="1"/>
+    <row r="461" ht="14.25" customHeight="1"/>
+    <row r="462" ht="14.25" customHeight="1"/>
+    <row r="463" ht="14.25" customHeight="1"/>
+    <row r="464" ht="14.25" customHeight="1"/>
+    <row r="465" ht="14.25" customHeight="1"/>
+    <row r="466" ht="14.25" customHeight="1"/>
+    <row r="467" ht="14.25" customHeight="1"/>
+    <row r="468" ht="14.25" customHeight="1"/>
+    <row r="469" ht="14.25" customHeight="1"/>
+    <row r="470" ht="14.25" customHeight="1"/>
+    <row r="471" ht="14.25" customHeight="1"/>
+    <row r="472" ht="14.25" customHeight="1"/>
+    <row r="473" ht="14.25" customHeight="1"/>
+    <row r="474" ht="14.25" customHeight="1"/>
+    <row r="475" ht="14.25" customHeight="1"/>
+    <row r="476" ht="14.25" customHeight="1"/>
+    <row r="477" ht="14.25" customHeight="1"/>
+    <row r="478" ht="14.25" customHeight="1"/>
+    <row r="479" ht="14.25" customHeight="1"/>
+    <row r="480" ht="14.25" customHeight="1"/>
+    <row r="481" ht="14.25" customHeight="1"/>
+    <row r="482" ht="14.25" customHeight="1"/>
+    <row r="483" ht="14.25" customHeight="1"/>
+    <row r="484" ht="14.25" customHeight="1"/>
+    <row r="485" ht="14.25" customHeight="1"/>
+    <row r="486" ht="14.25" customHeight="1"/>
+    <row r="487" ht="14.25" customHeight="1"/>
+    <row r="488" ht="14.25" customHeight="1"/>
+    <row r="489" ht="14.25" customHeight="1"/>
+    <row r="490" ht="14.25" customHeight="1"/>
+    <row r="491" ht="14.25" customHeight="1"/>
+    <row r="492" ht="14.25" customHeight="1"/>
+    <row r="493" ht="14.25" customHeight="1"/>
+    <row r="494" ht="14.25" customHeight="1"/>
+    <row r="495" ht="14.25" customHeight="1"/>
+    <row r="496" ht="14.25" customHeight="1"/>
+    <row r="497" ht="14.25" customHeight="1"/>
+    <row r="498" ht="14.25" customHeight="1"/>
+    <row r="499" ht="14.25" customHeight="1"/>
+    <row r="500" ht="14.25" customHeight="1"/>
+    <row r="501" ht="14.25" customHeight="1"/>
+    <row r="502" ht="14.25" customHeight="1"/>
+    <row r="503" ht="14.25" customHeight="1"/>
+    <row r="504" ht="14.25" customHeight="1"/>
+    <row r="505" ht="14.25" customHeight="1"/>
+    <row r="506" ht="14.25" customHeight="1"/>
+    <row r="507" ht="14.25" customHeight="1"/>
+    <row r="508" ht="14.25" customHeight="1"/>
+    <row r="509" ht="14.25" customHeight="1"/>
+    <row r="510" ht="14.25" customHeight="1"/>
+    <row r="511" ht="14.25" customHeight="1"/>
+    <row r="512" ht="14.25" customHeight="1"/>
+    <row r="513" ht="14.25" customHeight="1"/>
+    <row r="514" ht="14.25" customHeight="1"/>
+    <row r="515" ht="14.25" customHeight="1"/>
+    <row r="516" ht="14.25" customHeight="1"/>
+    <row r="517" ht="14.25" customHeight="1"/>
+    <row r="518" ht="14.25" customHeight="1"/>
+    <row r="519" ht="14.25" customHeight="1"/>
+    <row r="520" ht="14.25" customHeight="1"/>
+    <row r="521" ht="14.25" customHeight="1"/>
+    <row r="522" ht="14.25" customHeight="1"/>
+    <row r="523" ht="14.25" customHeight="1"/>
+    <row r="524" ht="14.25" customHeight="1"/>
+    <row r="525" ht="14.25" customHeight="1"/>
+    <row r="526" ht="14.25" customHeight="1"/>
+    <row r="527" ht="14.25" customHeight="1"/>
+    <row r="528" ht="14.25" customHeight="1"/>
+    <row r="529" ht="14.25" customHeight="1"/>
+    <row r="530" ht="14.25" customHeight="1"/>
+    <row r="531" ht="14.25" customHeight="1"/>
+    <row r="532" ht="14.25" customHeight="1"/>
+    <row r="533" ht="14.25" customHeight="1"/>
+    <row r="534" ht="14.25" customHeight="1"/>
+    <row r="535" ht="14.25" customHeight="1"/>
+    <row r="536" ht="14.25" customHeight="1"/>
+    <row r="537" ht="14.25" customHeight="1"/>
+    <row r="538" ht="14.25" customHeight="1"/>
+    <row r="539" ht="14.25" customHeight="1"/>
+    <row r="540" ht="14.25" customHeight="1"/>
+    <row r="541" ht="14.25" customHeight="1"/>
+    <row r="542" ht="14.25" customHeight="1"/>
+    <row r="543" ht="14.25" customHeight="1"/>
+    <row r="544" ht="14.25" customHeight="1"/>
+    <row r="545" ht="14.25" customHeight="1"/>
+    <row r="546" ht="14.25" customHeight="1"/>
+    <row r="547" ht="14.25" customHeight="1"/>
+    <row r="548" ht="14.25" customHeight="1"/>
+    <row r="549" ht="14.25" customHeight="1"/>
+    <row r="550" ht="14.25" customHeight="1"/>
+    <row r="551" ht="14.25" customHeight="1"/>
+    <row r="552" ht="14.25" customHeight="1"/>
+    <row r="553" ht="14.25" customHeight="1"/>
+    <row r="554" ht="14.25" customHeight="1"/>
+    <row r="555" ht="14.25" customHeight="1"/>
+    <row r="556" ht="14.25" customHeight="1"/>
+    <row r="557" ht="14.25" customHeight="1"/>
+    <row r="558" ht="14.25" customHeight="1"/>
+    <row r="559" ht="14.25" customHeight="1"/>
+    <row r="560" ht="14.25" customHeight="1"/>
+    <row r="561" ht="14.25" customHeight="1"/>
+    <row r="562" ht="14.25" customHeight="1"/>
+    <row r="563" ht="14.25" customHeight="1"/>
+    <row r="564" ht="14.25" customHeight="1"/>
+    <row r="565" ht="14.25" customHeight="1"/>
+    <row r="566" ht="14.25" customHeight="1"/>
+    <row r="567" ht="14.25" customHeight="1"/>
+    <row r="568" ht="14.25" customHeight="1"/>
+    <row r="569" ht="14.25" customHeight="1"/>
+    <row r="570" ht="14.25" customHeight="1"/>
+    <row r="571" ht="14.25" customHeight="1"/>
+    <row r="572" ht="14.25" customHeight="1"/>
+    <row r="573" ht="14.25" customHeight="1"/>
+    <row r="574" ht="14.25" customHeight="1"/>
+    <row r="575" ht="14.25" customHeight="1"/>
+    <row r="576" ht="14.25" customHeight="1"/>
+    <row r="577" ht="14.25" customHeight="1"/>
+    <row r="578" ht="14.25" customHeight="1"/>
+    <row r="579" ht="14.25" customHeight="1"/>
+    <row r="580" ht="14.25" customHeight="1"/>
+    <row r="581" ht="14.25" customHeight="1"/>
+    <row r="582" ht="14.25" customHeight="1"/>
+    <row r="583" ht="14.25" customHeight="1"/>
+    <row r="584" ht="14.25" customHeight="1"/>
+    <row r="585" ht="14.25" customHeight="1"/>
+    <row r="586" ht="14.25" customHeight="1"/>
+    <row r="587" ht="14.25" customHeight="1"/>
+    <row r="588" ht="14.25" customHeight="1"/>
+    <row r="589" ht="14.25" customHeight="1"/>
+    <row r="590" ht="14.25" customHeight="1"/>
+    <row r="591" ht="14.25" customHeight="1"/>
+    <row r="592" ht="14.25" customHeight="1"/>
+    <row r="593" ht="14.25" customHeight="1"/>
+    <row r="594" ht="14.25" customHeight="1"/>
+    <row r="595" ht="14.25" customHeight="1"/>
+    <row r="596" ht="14.25" customHeight="1"/>
+    <row r="597" ht="14.25" customHeight="1"/>
+    <row r="598" ht="14.25" customHeight="1"/>
+    <row r="599" ht="14.25" customHeight="1"/>
+    <row r="600" ht="14.25" customHeight="1"/>
+    <row r="601" ht="14.25" customHeight="1"/>
+    <row r="602" ht="14.25" customHeight="1"/>
+    <row r="603" ht="14.25" customHeight="1"/>
+    <row r="604" ht="14.25" customHeight="1"/>
+    <row r="605" ht="14.25" customHeight="1"/>
+    <row r="606" ht="14.25" customHeight="1"/>
+    <row r="607" ht="14.25" customHeight="1"/>
+    <row r="608" ht="14.25" customHeight="1"/>
+    <row r="609" ht="14.25" customHeight="1"/>
+    <row r="610" ht="14.25" customHeight="1"/>
+    <row r="611" ht="14.25" customHeight="1"/>
+    <row r="612" ht="14.25" customHeight="1"/>
+    <row r="613" ht="14.25" customHeight="1"/>
+    <row r="614" ht="14.25" customHeight="1"/>
+    <row r="615" ht="14.25" customHeight="1"/>
+    <row r="616" ht="14.25" customHeight="1"/>
+    <row r="617" ht="14.25" customHeight="1"/>
+    <row r="618" ht="14.25" customHeight="1"/>
+    <row r="619" ht="14.25" customHeight="1"/>
+    <row r="620" ht="14.25" customHeight="1"/>
+    <row r="621" ht="14.25" customHeight="1"/>
+    <row r="622" ht="14.25" customHeight="1"/>
+    <row r="623" ht="14.25" customHeight="1"/>
+    <row r="624" ht="14.25" customHeight="1"/>
+    <row r="625" ht="14.25" customHeight="1"/>
+    <row r="626" ht="14.25" customHeight="1"/>
+    <row r="627" ht="14.25" customHeight="1"/>
+    <row r="628" ht="14.25" customHeight="1"/>
+    <row r="629" ht="14.25" customHeight="1"/>
+    <row r="630" ht="14.25" customHeight="1"/>
+    <row r="631" ht="14.25" customHeight="1"/>
+    <row r="632" ht="14.25" customHeight="1"/>
+    <row r="633" ht="14.25" customHeight="1"/>
+    <row r="634" ht="14.25" customHeight="1"/>
+    <row r="635" ht="14.25" customHeight="1"/>
+    <row r="636" ht="14.25" customHeight="1"/>
+    <row r="637" ht="14.25" customHeight="1"/>
+    <row r="638" ht="14.25" customHeight="1"/>
+    <row r="639" ht="14.25" customHeight="1"/>
+    <row r="640" ht="14.25" customHeight="1"/>
+    <row r="641" ht="14.25" customHeight="1"/>
+    <row r="642" ht="14.25" customHeight="1"/>
+    <row r="643" ht="14.25" customHeight="1"/>
+    <row r="644" ht="14.25" customHeight="1"/>
+    <row r="645" ht="14.25" customHeight="1"/>
+    <row r="646" ht="14.25" customHeight="1"/>
+    <row r="647" ht="14.25" customHeight="1"/>
+    <row r="648" ht="14.25" customHeight="1"/>
+    <row r="649" ht="14.25" customHeight="1"/>
+    <row r="650" ht="14.25" customHeight="1"/>
+    <row r="651" ht="14.25" customHeight="1"/>
+    <row r="652" ht="14.25" customHeight="1"/>
+    <row r="653" ht="14.25" customHeight="1"/>
+    <row r="654" ht="14.25" customHeight="1"/>
+    <row r="655" ht="14.25" customHeight="1"/>
+    <row r="656" ht="14.25" customHeight="1"/>
+    <row r="657" ht="14.25" customHeight="1"/>
+    <row r="658" ht="14.25" customHeight="1"/>
+    <row r="659" ht="14.25" customHeight="1"/>
+    <row r="660" ht="14.25" customHeight="1"/>
+    <row r="661" ht="14.25" customHeight="1"/>
+    <row r="662" ht="14.25" customHeight="1"/>
+    <row r="663" ht="14.25" customHeight="1"/>
+    <row r="664" ht="14.25" customHeight="1"/>
+    <row r="665" ht="14.25" customHeight="1"/>
+    <row r="666" ht="14.25" customHeight="1"/>
+    <row r="667" ht="14.25" customHeight="1"/>
+    <row r="668" ht="14.25" customHeight="1"/>
+    <row r="669" ht="14.25" customHeight="1"/>
+    <row r="670" ht="14.25" customHeight="1"/>
+    <row r="671" ht="14.25" customHeight="1"/>
+    <row r="672" ht="14.25" customHeight="1"/>
+    <row r="673" ht="14.25" customHeight="1"/>
+    <row r="674" ht="14.25" customHeight="1"/>
+    <row r="675" ht="14.25" customHeight="1"/>
+    <row r="676" ht="14.25" customHeight="1"/>
+    <row r="677" ht="14.25" customHeight="1"/>
+    <row r="678" ht="14.25" customHeight="1"/>
+    <row r="679" ht="14.25" customHeight="1"/>
+    <row r="680" ht="14.25" customHeight="1"/>
+    <row r="681" ht="14.25" customHeight="1"/>
+    <row r="682" ht="14.25" customHeight="1"/>
+    <row r="683" ht="14.25" customHeight="1"/>
+    <row r="684" ht="14.25" customHeight="1"/>
+    <row r="685" ht="14.25" customHeight="1"/>
+    <row r="686" ht="14.25" customHeight="1"/>
+    <row r="687" ht="14.25" customHeight="1"/>
+    <row r="688" ht="14.25" customHeight="1"/>
+    <row r="689" ht="14.25" customHeight="1"/>
+    <row r="690" ht="14.25" customHeight="1"/>
+    <row r="691" ht="14.25" customHeight="1"/>
+    <row r="692" ht="14.25" customHeight="1"/>
+    <row r="693" ht="14.25" customHeight="1"/>
+    <row r="694" ht="14.25" customHeight="1"/>
+    <row r="695" ht="14.25" customHeight="1"/>
+    <row r="696" ht="14.25" customHeight="1"/>
+    <row r="697" ht="14.25" customHeight="1"/>
+    <row r="698" ht="14.25" customHeight="1"/>
+    <row r="699" ht="14.25" customHeight="1"/>
+    <row r="700" ht="14.25" customHeight="1"/>
+    <row r="701" ht="14.25" customHeight="1"/>
+    <row r="702" ht="14.25" customHeight="1"/>
+    <row r="703" ht="14.25" customHeight="1"/>
+    <row r="704" ht="14.25" customHeight="1"/>
+    <row r="705" ht="14.25" customHeight="1"/>
+    <row r="706" ht="14.25" customHeight="1"/>
+    <row r="707" ht="14.25" customHeight="1"/>
+    <row r="708" ht="14.25" customHeight="1"/>
+    <row r="709" ht="14.25" customHeight="1"/>
+    <row r="710" ht="14.25" customHeight="1"/>
+    <row r="711" ht="14.25" customHeight="1"/>
+    <row r="712" ht="14.25" customHeight="1"/>
+    <row r="713" ht="14.25" customHeight="1"/>
+    <row r="714" ht="14.25" customHeight="1"/>
+    <row r="715" ht="14.25" customHeight="1"/>
+    <row r="716" ht="14.25" customHeight="1"/>
+    <row r="717" ht="14.25" customHeight="1"/>
+    <row r="718" ht="14.25" customHeight="1"/>
+    <row r="719" ht="14.25" customHeight="1"/>
+    <row r="720" ht="14.25" customHeight="1"/>
+    <row r="721" ht="14.25" customHeight="1"/>
+    <row r="722" ht="14.25" customHeight="1"/>
+    <row r="723" ht="14.25" customHeight="1"/>
+    <row r="724" ht="14.25" customHeight="1"/>
+    <row r="725" ht="14.25" customHeight="1"/>
+    <row r="726" ht="14.25" customHeight="1"/>
+    <row r="727" ht="14.25" customHeight="1"/>
+    <row r="728" ht="14.25" customHeight="1"/>
+    <row r="729" ht="14.25" customHeight="1"/>
+    <row r="730" ht="14.25" customHeight="1"/>
+    <row r="731" ht="14.25" customHeight="1"/>
+    <row r="732" ht="14.25" customHeight="1"/>
+    <row r="733" ht="14.25" customHeight="1"/>
+    <row r="734" ht="14.25" customHeight="1"/>
+    <row r="735" ht="14.25" customHeight="1"/>
+    <row r="736" ht="14.25" customHeight="1"/>
+    <row r="737" ht="14.25" customHeight="1"/>
+    <row r="738" ht="14.25" customHeight="1"/>
+    <row r="739" ht="14.25" customHeight="1"/>
+    <row r="740" ht="14.25" customHeight="1"/>
+    <row r="741" ht="14.25" customHeight="1"/>
+    <row r="742" ht="14.25" customHeight="1"/>
+    <row r="743" ht="14.25" customHeight="1"/>
+    <row r="744" ht="14.25" customHeight="1"/>
+    <row r="745" ht="14.25" customHeight="1"/>
+    <row r="746" ht="14.25" customHeight="1"/>
+    <row r="747" ht="14.25" customHeight="1"/>
+    <row r="748" ht="14.25" customHeight="1"/>
+    <row r="749" ht="14.25" customHeight="1"/>
+    <row r="750" ht="14.25" customHeight="1"/>
+    <row r="751" ht="14.25" customHeight="1"/>
+    <row r="752" ht="14.25" customHeight="1"/>
+    <row r="753" ht="14.25" customHeight="1"/>
+    <row r="754" ht="14.25" customHeight="1"/>
+    <row r="755" ht="14.25" customHeight="1"/>
+    <row r="756" ht="14.25" customHeight="1"/>
+    <row r="757" ht="14.25" customHeight="1"/>
+    <row r="758" ht="14.25" customHeight="1"/>
+    <row r="759" ht="14.25" customHeight="1"/>
+    <row r="760" ht="14.25" customHeight="1"/>
+    <row r="761" ht="14.25" customHeight="1"/>
+    <row r="762" ht="14.25" customHeight="1"/>
+    <row r="763" ht="14.25" customHeight="1"/>
+    <row r="764" ht="14.25" customHeight="1"/>
+    <row r="765" ht="14.25" customHeight="1"/>
+    <row r="766" ht="14.25" customHeight="1"/>
+    <row r="767" ht="14.25" customHeight="1"/>
+    <row r="768" ht="14.25" customHeight="1"/>
+    <row r="769" ht="14.25" customHeight="1"/>
+    <row r="770" ht="14.25" customHeight="1"/>
+    <row r="771" ht="14.25" customHeight="1"/>
+    <row r="772" ht="14.25" customHeight="1"/>
+    <row r="773" ht="14.25" customHeight="1"/>
+    <row r="774" ht="14.25" customHeight="1"/>
+    <row r="775" ht="14.25" customHeight="1"/>
+    <row r="776" ht="14.25" customHeight="1"/>
+    <row r="777" ht="14.25" customHeight="1"/>
+    <row r="778" ht="14.25" customHeight="1"/>
+    <row r="779" ht="14.25" customHeight="1"/>
+    <row r="780" ht="14.25" customHeight="1"/>
+    <row r="781" ht="14.25" customHeight="1"/>
+    <row r="782" ht="14.25" customHeight="1"/>
+    <row r="783" ht="14.25" customHeight="1"/>
+    <row r="784" ht="14.25" customHeight="1"/>
+    <row r="785" ht="14.25" customHeight="1"/>
+    <row r="786" ht="14.25" customHeight="1"/>
+    <row r="787" ht="14.25" customHeight="1"/>
+    <row r="788" ht="14.25" customHeight="1"/>
+    <row r="789" ht="14.25" customHeight="1"/>
+    <row r="790" ht="14.25" customHeight="1"/>
+    <row r="791" ht="14.25" customHeight="1"/>
+    <row r="792" ht="14.25" customHeight="1"/>
+    <row r="793" ht="14.25" customHeight="1"/>
+    <row r="794" ht="14.25" customHeight="1"/>
+    <row r="795" ht="14.25" customHeight="1"/>
+    <row r="796" ht="14.25" customHeight="1"/>
+    <row r="797" ht="14.25" customHeight="1"/>
+    <row r="798" ht="14.25" customHeight="1"/>
+    <row r="799" ht="14.25" customHeight="1"/>
+    <row r="800" ht="14.25" customHeight="1"/>
+    <row r="801" ht="14.25" customHeight="1"/>
+    <row r="802" ht="14.25" customHeight="1"/>
+    <row r="803" ht="14.25" customHeight="1"/>
+    <row r="804" ht="14.25" customHeight="1"/>
+    <row r="805" ht="14.25" customHeight="1"/>
+    <row r="806" ht="14.25" customHeight="1"/>
+    <row r="807" ht="14.25" customHeight="1"/>
+    <row r="808" ht="14.25" customHeight="1"/>
+    <row r="809" ht="14.25" customHeight="1"/>
+    <row r="810" ht="14.25" customHeight="1"/>
+    <row r="811" ht="14.25" customHeight="1"/>
+    <row r="812" ht="14.25" customHeight="1"/>
+    <row r="813" ht="14.25" customHeight="1"/>
+    <row r="814" ht="14.25" customHeight="1"/>
+    <row r="815" ht="14.25" customHeight="1"/>
+    <row r="816" ht="14.25" customHeight="1"/>
+    <row r="817" ht="14.25" customHeight="1"/>
+    <row r="818" ht="14.25" customHeight="1"/>
+    <row r="819" ht="14.25" customHeight="1"/>
+    <row r="820" ht="14.25" customHeight="1"/>
+    <row r="821" ht="14.25" customHeight="1"/>
+    <row r="822" ht="14.25" customHeight="1"/>
+    <row r="823" ht="14.25" customHeight="1"/>
+    <row r="824" ht="14.25" customHeight="1"/>
+    <row r="825" ht="14.25" customHeight="1"/>
+    <row r="826" ht="14.25" customHeight="1"/>
+    <row r="827" ht="14.25" customHeight="1"/>
+    <row r="828" ht="14.25" customHeight="1"/>
+    <row r="829" ht="14.25" customHeight="1"/>
+    <row r="830" ht="14.25" customHeight="1"/>
+    <row r="831" ht="14.25" customHeight="1"/>
+    <row r="832" ht="14.25" customHeight="1"/>
+    <row r="833" ht="14.25" customHeight="1"/>
+    <row r="834" ht="14.25" customHeight="1"/>
+    <row r="835" ht="14.25" customHeight="1"/>
+    <row r="836" ht="14.25" customHeight="1"/>
+    <row r="837" ht="14.25" customHeight="1"/>
+    <row r="838" ht="14.25" customHeight="1"/>
+    <row r="839" ht="14.25" customHeight="1"/>
+    <row r="840" ht="14.25" customHeight="1"/>
+    <row r="841" ht="14.25" customHeight="1"/>
+    <row r="842" ht="14.25" customHeight="1"/>
+    <row r="843" ht="14.25" customHeight="1"/>
+    <row r="844" ht="14.25" customHeight="1"/>
+    <row r="845" ht="14.25" customHeight="1"/>
+    <row r="846" ht="14.25" customHeight="1"/>
+    <row r="847" ht="14.25" customHeight="1"/>
+    <row r="848" ht="14.25" customHeight="1"/>
+    <row r="849" ht="14.25" customHeight="1"/>
+    <row r="850" ht="14.25" customHeight="1"/>
+    <row r="851" ht="14.25" customHeight="1"/>
+    <row r="852" ht="14.25" customHeight="1"/>
+    <row r="853" ht="14.25" customHeight="1"/>
+    <row r="854" ht="14.25" customHeight="1"/>
+    <row r="855" ht="14.25" customHeight="1"/>
+    <row r="856" ht="14.25" customHeight="1"/>
+    <row r="857" ht="14.25" customHeight="1"/>
+    <row r="858" ht="14.25" customHeight="1"/>
+    <row r="859" ht="14.25" customHeight="1"/>
+    <row r="860" ht="14.25" customHeight="1"/>
+    <row r="861" ht="14.25" customHeight="1"/>
+    <row r="862" ht="14.25" customHeight="1"/>
+    <row r="863" ht="14.25" customHeight="1"/>
+    <row r="864" ht="14.25" customHeight="1"/>
+    <row r="865" ht="14.25" customHeight="1"/>
+    <row r="866" ht="14.25" customHeight="1"/>
+    <row r="867" ht="14.25" customHeight="1"/>
+    <row r="868" ht="14.25" customHeight="1"/>
+    <row r="869" ht="14.25" customHeight="1"/>
+    <row r="870" ht="14.25" customHeight="1"/>
+    <row r="871" ht="14.25" customHeight="1"/>
+    <row r="872" ht="14.25" customHeight="1"/>
+    <row r="873" ht="14.25" customHeight="1"/>
+    <row r="874" ht="14.25" customHeight="1"/>
+    <row r="875" ht="14.25" customHeight="1"/>
+    <row r="876" ht="14.25" customHeight="1"/>
+    <row r="877" ht="14.25" customHeight="1"/>
+    <row r="878" ht="14.25" customHeight="1"/>
+    <row r="879" ht="14.25" customHeight="1"/>
+    <row r="880" ht="14.25" customHeight="1"/>
+    <row r="881" ht="14.25" customHeight="1"/>
+    <row r="882" ht="14.25" customHeight="1"/>
+    <row r="883" ht="14.25" customHeight="1"/>
+    <row r="884" ht="14.25" customHeight="1"/>
+    <row r="885" ht="14.25" customHeight="1"/>
+    <row r="886" ht="14.25" customHeight="1"/>
+    <row r="887" ht="14.25" customHeight="1"/>
+    <row r="888" ht="14.25" customHeight="1"/>
+    <row r="889" ht="14.25" customHeight="1"/>
+    <row r="890" ht="14.25" customHeight="1"/>
+    <row r="891" ht="14.25" customHeight="1"/>
+    <row r="892" ht="14.25" customHeight="1"/>
+    <row r="893" ht="14.25" customHeight="1"/>
+    <row r="894" ht="14.25" customHeight="1"/>
+    <row r="895" ht="14.25" customHeight="1"/>
+    <row r="896" ht="14.25" customHeight="1"/>
+    <row r="897" ht="14.25" customHeight="1"/>
+    <row r="898" ht="14.25" customHeight="1"/>
+    <row r="899" ht="14.25" customHeight="1"/>
+    <row r="900" ht="14.25" customHeight="1"/>
+    <row r="901" ht="14.25" customHeight="1"/>
+    <row r="902" ht="14.25" customHeight="1"/>
+    <row r="903" ht="14.25" customHeight="1"/>
+    <row r="904" ht="14.25" customHeight="1"/>
+    <row r="905" ht="14.25" customHeight="1"/>
+    <row r="906" ht="14.25" customHeight="1"/>
+    <row r="907" ht="14.25" customHeight="1"/>
+    <row r="908" ht="14.25" customHeight="1"/>
+    <row r="909" ht="14.25" customHeight="1"/>
+    <row r="910" ht="14.25" customHeight="1"/>
+    <row r="911" ht="14.25" customHeight="1"/>
+    <row r="912" ht="14.25" customHeight="1"/>
+    <row r="913" ht="14.25" customHeight="1"/>
+    <row r="914" ht="14.25" customHeight="1"/>
+    <row r="915" ht="14.25" customHeight="1"/>
+    <row r="916" ht="14.25" customHeight="1"/>
+    <row r="917" ht="14.25" customHeight="1"/>
+    <row r="918" ht="14.25" customHeight="1"/>
+    <row r="919" ht="14.25" customHeight="1"/>
+    <row r="920" ht="14.25" customHeight="1"/>
+    <row r="921" ht="14.25" customHeight="1"/>
+    <row r="922" ht="14.25" customHeight="1"/>
+    <row r="923" ht="14.25" customHeight="1"/>
+    <row r="924" ht="14.25" customHeight="1"/>
+    <row r="925" ht="14.25" customHeight="1"/>
+    <row r="926" ht="14.25" customHeight="1"/>
+    <row r="927" ht="14.25" customHeight="1"/>
+    <row r="928" ht="14.25" customHeight="1"/>
+    <row r="929" ht="14.25" customHeight="1"/>
+    <row r="930" ht="14.25" customHeight="1"/>
+    <row r="931" ht="14.25" customHeight="1"/>
+    <row r="932" ht="14.25" customHeight="1"/>
+    <row r="933" ht="14.25" customHeight="1"/>
+    <row r="934" ht="14.25" customHeight="1"/>
+    <row r="935" ht="14.25" customHeight="1"/>
+    <row r="936" ht="14.25" customHeight="1"/>
+    <row r="937" ht="14.25" customHeight="1"/>
+    <row r="938" ht="14.25" customHeight="1"/>
+    <row r="939" ht="14.25" customHeight="1"/>
+    <row r="940" ht="14.25" customHeight="1"/>
+    <row r="941" ht="14.25" customHeight="1"/>
+    <row r="942" ht="14.25" customHeight="1"/>
+    <row r="943" ht="14.25" customHeight="1"/>
+    <row r="944" ht="14.25" customHeight="1"/>
+    <row r="945" ht="14.25" customHeight="1"/>
+    <row r="946" ht="14.25" customHeight="1"/>
+    <row r="947" ht="14.25" customHeight="1"/>
+    <row r="948" ht="14.25" customHeight="1"/>
+    <row r="949" ht="14.25" customHeight="1"/>
+    <row r="950" ht="14.25" customHeight="1"/>
+    <row r="951" ht="14.25" customHeight="1"/>
+    <row r="952" ht="14.25" customHeight="1"/>
+    <row r="953" ht="14.25" customHeight="1"/>
+    <row r="954" ht="14.25" customHeight="1"/>
+    <row r="955" ht="14.25" customHeight="1"/>
+    <row r="956" ht="14.25" customHeight="1"/>
+    <row r="957" ht="14.25" customHeight="1"/>
+    <row r="958" ht="14.25" customHeight="1"/>
+    <row r="959" ht="14.25" customHeight="1"/>
+    <row r="960" ht="14.25" customHeight="1"/>
+    <row r="961" ht="14.25" customHeight="1"/>
+    <row r="962" ht="14.25" customHeight="1"/>
+    <row r="963" ht="14.25" customHeight="1"/>
+    <row r="964" ht="14.25" customHeight="1"/>
+    <row r="965" ht="14.25" customHeight="1"/>
+    <row r="966" ht="14.25" customHeight="1"/>
+    <row r="967" ht="14.25" customHeight="1"/>
+    <row r="968" ht="14.25" customHeight="1"/>
+    <row r="969" ht="14.25" customHeight="1"/>
+    <row r="970" ht="14.25" customHeight="1"/>
+    <row r="971" ht="14.25" customHeight="1"/>
+    <row r="972" ht="14.25" customHeight="1"/>
+    <row r="973" ht="14.25" customHeight="1"/>
+    <row r="974" ht="14.25" customHeight="1"/>
+    <row r="975" ht="14.25" customHeight="1"/>
+    <row r="976" ht="14.25" customHeight="1"/>
+    <row r="977" ht="14.25" customHeight="1"/>
+    <row r="978" ht="14.25" customHeight="1"/>
+    <row r="979" ht="14.25" customHeight="1"/>
+    <row r="980" ht="14.25" customHeight="1"/>
+    <row r="981" ht="14.25" customHeight="1"/>
+    <row r="982" ht="14.25" customHeight="1"/>
+    <row r="983" ht="14.25" customHeight="1"/>
+    <row r="984" ht="14.25" customHeight="1"/>
+    <row r="985" ht="14.25" customHeight="1"/>
+    <row r="986" ht="14.25" customHeight="1"/>
+    <row r="987" ht="14.25" customHeight="1"/>
+    <row r="988" ht="14.25" customHeight="1"/>
+    <row r="989" ht="14.25" customHeight="1"/>
+    <row r="990" ht="14.25" customHeight="1"/>
+    <row r="991" ht="14.25" customHeight="1"/>
+    <row r="992" ht="14.25" customHeight="1"/>
+    <row r="993" ht="14.25" customHeight="1"/>
+    <row r="994" ht="14.25" customHeight="1"/>
+    <row r="995" ht="14.25" customHeight="1"/>
+    <row r="996" ht="14.25" customHeight="1"/>
+    <row r="997" ht="14.25" customHeight="1"/>
+    <row r="998" ht="14.25" customHeight="1"/>
+    <row r="999" ht="14.25" customHeight="1"/>
+    <row r="1000" ht="14.25" customHeight="1"/>
+    <row r="1001" ht="14.25" customHeight="1"/>
+    <row r="1002" ht="14.25" customHeight="1"/>
+  </sheetData>
+  <printOptions/>
+  <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <pageSetUpPr/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <cols>
     <col customWidth="1" min="1" max="1" width="28.0"/>
     <col customWidth="1" min="2" max="3" width="22.0"/>
     <col customWidth="1" min="4" max="4" width="14.0"/>
@@ -5206,173 +7116,173 @@
   </cols>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="15" t="s">
-        <v>127</v>
+      <c r="A1" s="54" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>128</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1"/>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>129</v>
+        <v>165</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>130</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>131</v>
+        <v>167</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>132</v>
+        <v>168</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1"/>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="48" t="s">
-        <v>133</v>
-      </c>
-      <c r="B7" s="48" t="s">
-        <v>134</v>
-      </c>
-      <c r="C7" s="48" t="s">
-        <v>135</v>
-      </c>
-      <c r="D7" s="48" t="s">
-        <v>136</v>
-      </c>
-      <c r="E7" s="48" t="s">
-        <v>137</v>
+      <c r="A7" s="55" t="s">
+        <v>169</v>
+      </c>
+      <c r="B7" s="55" t="s">
+        <v>170</v>
+      </c>
+      <c r="C7" s="55" t="s">
+        <v>171</v>
+      </c>
+      <c r="D7" s="55" t="s">
+        <v>172</v>
+      </c>
+      <c r="E7" s="55" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
-      <c r="A8" s="49" t="s">
-        <v>138</v>
-      </c>
-      <c r="B8" s="50">
+      <c r="A8" s="56" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" s="57">
         <v>18.0</v>
       </c>
-      <c r="C8" s="50">
+      <c r="C8" s="57">
         <v>18.0</v>
       </c>
-      <c r="D8" s="50">
+      <c r="D8" s="57">
         <v>0.0</v>
       </c>
-      <c r="E8" s="18" t="s">
-        <v>139</v>
+      <c r="E8" s="19" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="9" ht="24.75" customHeight="1">
-      <c r="A9" s="49" t="s">
-        <v>140</v>
-      </c>
-      <c r="B9" s="50">
+      <c r="A9" s="56" t="s">
+        <v>176</v>
+      </c>
+      <c r="B9" s="57">
         <v>13.5</v>
       </c>
-      <c r="C9" s="50" t="s">
-        <v>141</v>
-      </c>
-      <c r="D9" s="50"/>
-      <c r="E9" s="18" t="s">
-        <v>142</v>
+      <c r="C9" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="D9" s="57"/>
+      <c r="E9" s="19" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="10" ht="24.75" customHeight="1">
-      <c r="A10" s="49" t="s">
-        <v>143</v>
-      </c>
-      <c r="B10" s="50">
+      <c r="A10" s="56" t="s">
+        <v>179</v>
+      </c>
+      <c r="B10" s="57">
         <v>9.0</v>
       </c>
-      <c r="C10" s="50" t="s">
-        <v>141</v>
-      </c>
-      <c r="D10" s="50"/>
-      <c r="E10" s="18" t="s">
-        <v>144</v>
+      <c r="C10" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="D10" s="57"/>
+      <c r="E10" s="19" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="11" ht="24.75" customHeight="1">
-      <c r="A11" s="49" t="s">
-        <v>145</v>
-      </c>
-      <c r="B11" s="50">
+      <c r="A11" s="56" t="s">
+        <v>181</v>
+      </c>
+      <c r="B11" s="57">
         <v>4.5</v>
       </c>
-      <c r="C11" s="50" t="s">
-        <v>141</v>
-      </c>
-      <c r="D11" s="50"/>
-      <c r="E11" s="18" t="s">
-        <v>146</v>
+      <c r="C11" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="D11" s="57"/>
+      <c r="E11" s="19" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="12" ht="24.75" customHeight="1">
-      <c r="A12" s="49" t="s">
-        <v>147</v>
-      </c>
-      <c r="B12" s="50">
+      <c r="A12" s="56" t="s">
+        <v>183</v>
+      </c>
+      <c r="B12" s="57">
         <v>0.0</v>
       </c>
-      <c r="C12" s="50" t="s">
-        <v>141</v>
-      </c>
-      <c r="D12" s="50"/>
-      <c r="E12" s="18" t="s">
-        <v>148</v>
+      <c r="C12" s="57" t="s">
+        <v>177</v>
+      </c>
+      <c r="D12" s="57"/>
+      <c r="E12" s="19" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1"/>
     <row r="14" ht="14.25" customHeight="1"/>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>149</v>
+        <v>185</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>150</v>
+        <v>186</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="3" t="s">
-        <v>151</v>
+        <v>187</v>
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="A18" s="19" t="s">
-        <v>152</v>
+      <c r="A18" s="20" t="s">
+        <v>188</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>153</v>
+        <v>189</v>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="47" t="s">
-        <v>154</v>
+      <c r="A19" s="53" t="s">
+        <v>190</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>155</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" s="19" t="s">
-        <v>156</v>
+      <c r="A20" s="20" t="s">
+        <v>192</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>157</v>
+        <v>193</v>
       </c>
     </row>
     <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" s="20" t="s">
-        <v>158</v>
+      <c r="A21" s="21" t="s">
+        <v>194</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>159</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" ht="14.25" customHeight="1"/>
@@ -6362,7 +8272,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <pageSetUpPr/>
@@ -6379,135 +8289,135 @@
     <row r="1" ht="14.25" customHeight="1"/>
     <row r="2" ht="14.25" customHeight="1">
       <c r="B2" s="2" t="s">
-        <v>160</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="B3" s="9" t="s">
-        <v>161</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1"/>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="48"/>
-      <c r="B5" s="48" t="s">
-        <v>162</v>
-      </c>
-      <c r="C5" s="48" t="s">
-        <v>163</v>
-      </c>
-      <c r="D5" s="51" t="s">
-        <v>164</v>
+      <c r="A5" s="55"/>
+      <c r="B5" s="55" t="s">
+        <v>198</v>
+      </c>
+      <c r="C5" s="55" t="s">
+        <v>199</v>
+      </c>
+      <c r="D5" s="58" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="6" ht="30.0" customHeight="1">
-      <c r="B6" s="52" t="s">
-        <v>165</v>
-      </c>
-      <c r="C6" s="53" t="s">
-        <v>166</v>
-      </c>
-      <c r="D6" s="52" t="s">
-        <v>167</v>
+      <c r="B6" s="59" t="s">
+        <v>201</v>
+      </c>
+      <c r="C6" s="60" t="s">
+        <v>202</v>
+      </c>
+      <c r="D6" s="59" t="s">
+        <v>203</v>
       </c>
     </row>
     <row r="7" ht="30.0" customHeight="1">
-      <c r="B7" s="52" t="s">
-        <v>168</v>
-      </c>
-      <c r="C7" s="53" t="s">
-        <v>169</v>
-      </c>
-      <c r="D7" s="52" t="s">
-        <v>170</v>
+      <c r="B7" s="59" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="60" t="s">
+        <v>205</v>
+      </c>
+      <c r="D7" s="59" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="8" ht="30.0" customHeight="1">
-      <c r="B8" s="52" t="s">
-        <v>171</v>
-      </c>
-      <c r="C8" s="53" t="s">
-        <v>172</v>
-      </c>
-      <c r="D8" s="52" t="s">
-        <v>173</v>
+      <c r="B8" s="59" t="s">
+        <v>207</v>
+      </c>
+      <c r="C8" s="60" t="s">
+        <v>208</v>
+      </c>
+      <c r="D8" s="59" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="9" ht="30.0" customHeight="1">
-      <c r="B9" s="52" t="s">
-        <v>174</v>
-      </c>
-      <c r="C9" s="53" t="s">
-        <v>169</v>
-      </c>
-      <c r="D9" s="52" t="s">
-        <v>175</v>
+      <c r="B9" s="59" t="s">
+        <v>210</v>
+      </c>
+      <c r="C9" s="60" t="s">
+        <v>205</v>
+      </c>
+      <c r="D9" s="59" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="10" ht="30.0" customHeight="1">
-      <c r="B10" s="52" t="s">
-        <v>176</v>
-      </c>
-      <c r="C10" s="53" t="s">
-        <v>177</v>
-      </c>
-      <c r="D10" s="52" t="s">
-        <v>178</v>
+      <c r="B10" s="59" t="s">
+        <v>212</v>
+      </c>
+      <c r="C10" s="60" t="s">
+        <v>213</v>
+      </c>
+      <c r="D10" s="59" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="11" ht="30.0" customHeight="1">
-      <c r="B11" s="52" t="s">
-        <v>179</v>
-      </c>
-      <c r="C11" s="53" t="s">
-        <v>177</v>
-      </c>
-      <c r="D11" s="54" t="s">
-        <v>180</v>
+      <c r="B11" s="59" t="s">
+        <v>215</v>
+      </c>
+      <c r="C11" s="60" t="s">
+        <v>213</v>
+      </c>
+      <c r="D11" s="61" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="12" ht="30.0" customHeight="1">
-      <c r="B12" s="52" t="s">
-        <v>181</v>
-      </c>
-      <c r="C12" s="53" t="s">
-        <v>177</v>
-      </c>
-      <c r="D12" s="52" t="s">
-        <v>182</v>
+      <c r="B12" s="59" t="s">
+        <v>217</v>
+      </c>
+      <c r="C12" s="60" t="s">
+        <v>213</v>
+      </c>
+      <c r="D12" s="59" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="13" ht="30.0" customHeight="1">
-      <c r="B13" s="52" t="s">
-        <v>183</v>
-      </c>
-      <c r="C13" s="53" t="s">
-        <v>184</v>
-      </c>
-      <c r="D13" s="52" t="s">
-        <v>185</v>
+      <c r="B13" s="59" t="s">
+        <v>219</v>
+      </c>
+      <c r="C13" s="60" t="s">
+        <v>220</v>
+      </c>
+      <c r="D13" s="59" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="14" ht="30.0" customHeight="1">
-      <c r="B14" s="52" t="s">
-        <v>186</v>
-      </c>
-      <c r="C14" s="53" t="s">
-        <v>177</v>
-      </c>
-      <c r="D14" s="52" t="s">
-        <v>187</v>
+      <c r="B14" s="59" t="s">
+        <v>222</v>
+      </c>
+      <c r="C14" s="60" t="s">
+        <v>213</v>
+      </c>
+      <c r="D14" s="59" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="15" ht="30.0" customHeight="1">
-      <c r="B15" s="52" t="s">
-        <v>188</v>
-      </c>
-      <c r="C15" s="55" t="s">
-        <v>189</v>
-      </c>
-      <c r="D15" s="52" t="s">
-        <v>190</v>
+      <c r="B15" s="59" t="s">
+        <v>224</v>
+      </c>
+      <c r="C15" s="62" t="s">
+        <v>225</v>
+      </c>
+      <c r="D15" s="59" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
docs: update sprint backlog burndown burnup
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-25-sprint-backlog-v1.0.xlsx
+++ b/docs/cadrage/equipe-25-sprint-backlog-v1.0.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="231">
   <si>
     <t>A</t>
   </si>
@@ -554,9 +554,6 @@
     <t>15h00, Daily intermédiaire</t>
   </si>
   <si>
-    <t>[à compléter]</t>
-  </si>
-  <si>
     <t>1/4 du sprint écoulé</t>
   </si>
   <si>
@@ -609,6 +606,21 @@
   </si>
   <si>
     <t>Tâches bloquées, escalader immédiatement avec le Scrum Master</t>
+  </si>
+  <si>
+    <t>Le BURNUP trace le travail livré cumulé pendant le sprint.</t>
+  </si>
+  <si>
+    <t>Moment</t>
+  </si>
+  <si>
+    <t>Travail livré idéal</t>
+  </si>
+  <si>
+    <t>Travail livré réel</t>
+  </si>
+  <si>
+    <t>Scope total</t>
   </si>
   <si>
     <t>✅ Grille d'auto-évaluation</t>
@@ -708,7 +720,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -831,7 +843,6 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -861,6 +872,12 @@
     </font>
     <font>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -1003,7 +1020,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="58">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1021,20 +1038,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="2" fillId="2" fontId="14" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1052,9 +1058,6 @@
     <xf borderId="4" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="4" fillId="4" fontId="19" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="4" fontId="20" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="4" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1066,34 +1069,25 @@
     <xf borderId="4" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="4" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="0" fillId="6" fontId="20" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="4" fillId="5" fontId="19" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="5" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="5" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="6" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="6" fillId="5" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="6" fillId="5" fontId="21" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -1101,9 +1095,7 @@
     <xf borderId="6" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
-    <xf borderId="6" fillId="5" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="6" fillId="5" fontId="23" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="5" fontId="22" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1112,15 +1104,9 @@
     </xf>
     <xf borderId="7" fillId="7" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="7" fillId="7" fontId="23" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="7" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="7" fillId="7" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="7" fillId="7" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="24" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="25" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -1128,20 +1114,32 @@
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="26" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="26" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="6" fillId="3" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="27" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="6" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="15" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="20" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="23" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2462,7 +2460,7 @@
       <c r="B7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="12" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2470,7 +2468,7 @@
       <c r="B8" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="12" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2478,7 +2476,7 @@
       <c r="B9" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="12" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2486,13 +2484,13 @@
       <c r="B10" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="12" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1"/>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="13" t="s">
         <v>20</v>
       </c>
     </row>
@@ -3513,12 +3511,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="23.25" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="9" t="s">
         <v>23</v>
       </c>
     </row>
@@ -3529,66 +3527,66 @@
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="16" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" ht="27.75" customHeight="1">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="16" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="16" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" ht="30.0" customHeight="1">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="16" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="10" ht="81.0" customHeight="1">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="16" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="16" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="16" t="s">
         <v>40</v>
       </c>
     </row>
@@ -3610,7 +3608,7 @@
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="17" t="s">
         <v>45</v>
       </c>
       <c r="B16" s="9" t="s">
@@ -3618,7 +3616,7 @@
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B17" s="9" t="s">
@@ -3627,1013 +3625,1013 @@
     </row>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="22" t="s">
+      <c r="D19" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="F19" s="22" t="s">
+      <c r="F19" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="G19" s="22" t="s">
+      <c r="G19" s="19" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" ht="30.0" customHeight="1">
-      <c r="A20" s="23" t="s">
+      <c r="A20" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="D20" s="24" t="s">
+      <c r="D20" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="E20" s="25">
+      <c r="E20" s="22">
         <v>1.0</v>
       </c>
-      <c r="F20" s="25">
+      <c r="F20" s="22">
         <v>1.0</v>
       </c>
-      <c r="G20" s="24" t="s">
+      <c r="G20" s="21" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="21" ht="30.0" customHeight="1">
-      <c r="A21" s="23" t="s">
+      <c r="A21" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="20" t="s">
         <v>60</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="21" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="24" t="s">
+      <c r="D21" s="21" t="s">
         <v>62</v>
       </c>
-      <c r="E21" s="25">
+      <c r="E21" s="22">
         <v>2.0</v>
       </c>
-      <c r="F21" s="25">
+      <c r="F21" s="22">
         <v>2.0</v>
       </c>
-      <c r="G21" s="24" t="s">
+      <c r="G21" s="21" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="22" ht="30.0" customHeight="1">
-      <c r="A22" s="23" t="s">
+      <c r="A22" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="E22" s="25">
+      <c r="E22" s="22">
         <v>3.0</v>
       </c>
-      <c r="F22" s="25">
+      <c r="F22" s="22">
         <v>3.0</v>
       </c>
-      <c r="G22" s="24" t="s">
+      <c r="G22" s="21" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="23" ht="30.0" customHeight="1">
-      <c r="A23" s="23" t="s">
+      <c r="A23" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="D23" s="24" t="s">
+      <c r="D23" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="E23" s="25">
+      <c r="E23" s="22">
         <v>1.0</v>
       </c>
-      <c r="F23" s="25">
+      <c r="F23" s="22">
         <v>1.0</v>
       </c>
-      <c r="G23" s="26" t="s">
+      <c r="G23" s="21" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="24" ht="30.0" customHeight="1">
-      <c r="A24" s="27" t="s">
+      <c r="A24" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="B24" s="27" t="s">
+      <c r="B24" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="D24" s="24" t="s">
+      <c r="D24" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="25">
+      <c r="E24" s="22">
         <v>1.0</v>
       </c>
-      <c r="F24" s="25">
+      <c r="F24" s="22">
         <v>1.0</v>
       </c>
-      <c r="G24" s="24" t="s">
+      <c r="G24" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="H24" s="28"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="28"/>
-      <c r="K24" s="28"/>
-      <c r="L24" s="28"/>
-      <c r="M24" s="28"/>
-      <c r="N24" s="28"/>
-      <c r="O24" s="28"/>
-      <c r="P24" s="28"/>
-      <c r="Q24" s="28"/>
-      <c r="R24" s="28"/>
-      <c r="S24" s="28"/>
-      <c r="T24" s="28"/>
-      <c r="U24" s="28"/>
-      <c r="V24" s="28"/>
-      <c r="W24" s="28"/>
-      <c r="X24" s="28"/>
-      <c r="Y24" s="28"/>
-      <c r="Z24" s="28"/>
+      <c r="H24" s="24"/>
+      <c r="I24" s="24"/>
+      <c r="J24" s="24"/>
+      <c r="K24" s="24"/>
+      <c r="L24" s="24"/>
+      <c r="M24" s="24"/>
+      <c r="N24" s="24"/>
+      <c r="O24" s="24"/>
+      <c r="P24" s="24"/>
+      <c r="Q24" s="24"/>
+      <c r="R24" s="24"/>
+      <c r="S24" s="24"/>
+      <c r="T24" s="24"/>
+      <c r="U24" s="24"/>
+      <c r="V24" s="24"/>
+      <c r="W24" s="24"/>
+      <c r="X24" s="24"/>
+      <c r="Y24" s="24"/>
+      <c r="Z24" s="24"/>
     </row>
     <row r="25" ht="30.0" customHeight="1">
-      <c r="A25" s="29" t="s">
+      <c r="A25" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="C25" s="30" t="s">
+      <c r="C25" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="D25" s="30" t="s">
+      <c r="D25" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="E25" s="31">
+      <c r="E25" s="27">
         <v>1.0</v>
       </c>
-      <c r="F25" s="31">
+      <c r="F25" s="27">
         <v>1.0</v>
       </c>
-      <c r="G25" s="30" t="s">
+      <c r="G25" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="26" ht="30.0" customHeight="1">
-      <c r="A26" s="29" t="s">
+      <c r="A26" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B26" s="29" t="s">
+      <c r="B26" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="C26" s="30" t="s">
+      <c r="C26" s="26" t="s">
         <v>76</v>
       </c>
-      <c r="D26" s="30" t="s">
+      <c r="D26" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="E26" s="31">
+      <c r="E26" s="27">
         <v>3.0</v>
       </c>
-      <c r="F26" s="31">
+      <c r="F26" s="27">
         <v>3.0</v>
       </c>
-      <c r="G26" s="30" t="s">
+      <c r="G26" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="27" ht="30.0" customHeight="1">
-      <c r="A27" s="29" t="s">
+      <c r="A27" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B27" s="29" t="s">
+      <c r="B27" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="C27" s="30" t="s">
+      <c r="C27" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="D27" s="30" t="s">
+      <c r="D27" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="E27" s="31">
+      <c r="E27" s="27">
         <v>1.0</v>
       </c>
-      <c r="F27" s="32">
+      <c r="F27" s="27">
         <v>0.0</v>
       </c>
-      <c r="G27" s="33" t="s">
+      <c r="G27" s="26" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="28" ht="30.0" customHeight="1">
-      <c r="A28" s="29" t="s">
+      <c r="A28" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B28" s="29" t="s">
+      <c r="B28" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="C28" s="30" t="s">
+      <c r="C28" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="D28" s="30" t="s">
+      <c r="D28" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="E28" s="31">
+      <c r="E28" s="27">
         <v>3.0</v>
       </c>
-      <c r="F28" s="31">
+      <c r="F28" s="27">
         <v>3.0</v>
       </c>
-      <c r="G28" s="30" t="s">
+      <c r="G28" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="29" ht="30.0" customHeight="1">
-      <c r="A29" s="29" t="s">
+      <c r="A29" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B29" s="29" t="s">
+      <c r="B29" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="C29" s="30" t="s">
+      <c r="C29" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="D29" s="30" t="s">
+      <c r="D29" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="E29" s="31">
+      <c r="E29" s="27">
         <v>1.0</v>
       </c>
-      <c r="F29" s="32">
+      <c r="F29" s="27">
         <v>0.0</v>
       </c>
-      <c r="G29" s="33" t="s">
+      <c r="G29" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
-      <c r="K29" s="34"/>
-      <c r="L29" s="34"/>
-      <c r="M29" s="34"/>
-      <c r="N29" s="34"/>
-      <c r="O29" s="34"/>
-      <c r="P29" s="34"/>
-      <c r="Q29" s="34"/>
-      <c r="R29" s="34"/>
-      <c r="S29" s="34"/>
-      <c r="T29" s="34"/>
-      <c r="U29" s="34"/>
-      <c r="V29" s="34"/>
-      <c r="W29" s="34"/>
-      <c r="X29" s="34"/>
-      <c r="Y29" s="34"/>
-      <c r="Z29" s="34"/>
+      <c r="H29" s="28"/>
+      <c r="I29" s="28"/>
+      <c r="J29" s="28"/>
+      <c r="K29" s="28"/>
+      <c r="L29" s="28"/>
+      <c r="M29" s="28"/>
+      <c r="N29" s="28"/>
+      <c r="O29" s="28"/>
+      <c r="P29" s="28"/>
+      <c r="Q29" s="28"/>
+      <c r="R29" s="28"/>
+      <c r="S29" s="28"/>
+      <c r="T29" s="28"/>
+      <c r="U29" s="28"/>
+      <c r="V29" s="28"/>
+      <c r="W29" s="28"/>
+      <c r="X29" s="28"/>
+      <c r="Y29" s="28"/>
+      <c r="Z29" s="28"/>
     </row>
     <row r="30" ht="30.0" customHeight="1">
-      <c r="A30" s="35" t="s">
+      <c r="A30" s="29" t="s">
         <v>72</v>
       </c>
-      <c r="B30" s="35" t="s">
+      <c r="B30" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="C30" s="30" t="s">
+      <c r="C30" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="D30" s="30" t="s">
+      <c r="D30" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="E30" s="31">
+      <c r="E30" s="27">
         <v>1.0</v>
       </c>
-      <c r="F30" s="31">
+      <c r="F30" s="27">
         <v>1.0</v>
       </c>
-      <c r="G30" s="30" t="s">
+      <c r="G30" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="H30" s="34"/>
-      <c r="I30" s="34"/>
-      <c r="J30" s="34"/>
-      <c r="K30" s="34"/>
-      <c r="L30" s="34"/>
-      <c r="M30" s="34"/>
-      <c r="N30" s="34"/>
-      <c r="O30" s="34"/>
-      <c r="P30" s="34"/>
-      <c r="Q30" s="34"/>
-      <c r="R30" s="34"/>
-      <c r="S30" s="34"/>
-      <c r="T30" s="34"/>
-      <c r="U30" s="34"/>
-      <c r="V30" s="34"/>
-      <c r="W30" s="34"/>
-      <c r="X30" s="34"/>
-      <c r="Y30" s="34"/>
-      <c r="Z30" s="34"/>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="28"/>
+      <c r="K30" s="28"/>
+      <c r="L30" s="28"/>
+      <c r="M30" s="28"/>
+      <c r="N30" s="28"/>
+      <c r="O30" s="28"/>
+      <c r="P30" s="28"/>
+      <c r="Q30" s="28"/>
+      <c r="R30" s="28"/>
+      <c r="S30" s="28"/>
+      <c r="T30" s="28"/>
+      <c r="U30" s="28"/>
+      <c r="V30" s="28"/>
+      <c r="W30" s="28"/>
+      <c r="X30" s="28"/>
+      <c r="Y30" s="28"/>
+      <c r="Z30" s="28"/>
     </row>
     <row r="31" ht="30.0" customHeight="1">
-      <c r="A31" s="36" t="s">
+      <c r="A31" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B31" s="36" t="s">
+      <c r="B31" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="C31" s="33" t="s">
+      <c r="C31" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="E31" s="32">
+      <c r="E31" s="27">
         <v>1.0</v>
       </c>
-      <c r="F31" s="32">
+      <c r="F31" s="27">
         <v>1.0</v>
       </c>
-      <c r="G31" s="33" t="s">
+      <c r="G31" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="H31" s="34"/>
-      <c r="I31" s="34"/>
-      <c r="J31" s="34"/>
-      <c r="K31" s="34"/>
-      <c r="L31" s="34"/>
-      <c r="M31" s="34"/>
-      <c r="N31" s="34"/>
-      <c r="O31" s="34"/>
-      <c r="P31" s="34"/>
-      <c r="Q31" s="34"/>
-      <c r="R31" s="34"/>
-      <c r="S31" s="34"/>
-      <c r="T31" s="34"/>
-      <c r="U31" s="34"/>
-      <c r="V31" s="34"/>
-      <c r="W31" s="34"/>
-      <c r="X31" s="34"/>
-      <c r="Y31" s="34"/>
-      <c r="Z31" s="34"/>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="28"/>
+      <c r="K31" s="28"/>
+      <c r="L31" s="28"/>
+      <c r="M31" s="28"/>
+      <c r="N31" s="28"/>
+      <c r="O31" s="28"/>
+      <c r="P31" s="28"/>
+      <c r="Q31" s="28"/>
+      <c r="R31" s="28"/>
+      <c r="S31" s="28"/>
+      <c r="T31" s="28"/>
+      <c r="U31" s="28"/>
+      <c r="V31" s="28"/>
+      <c r="W31" s="28"/>
+      <c r="X31" s="28"/>
+      <c r="Y31" s="28"/>
+      <c r="Z31" s="28"/>
     </row>
     <row r="32" ht="30.0" customHeight="1">
-      <c r="A32" s="36" t="s">
+      <c r="A32" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B32" s="36" t="s">
+      <c r="B32" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="C32" s="33" t="s">
+      <c r="C32" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="E32" s="32">
+      <c r="E32" s="27">
         <v>1.0</v>
       </c>
-      <c r="F32" s="32">
+      <c r="F32" s="27">
         <v>1.0</v>
       </c>
-      <c r="G32" s="33" t="s">
+      <c r="G32" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="33" ht="30.0" customHeight="1">
-      <c r="A33" s="36" t="s">
+      <c r="A33" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B33" s="36" t="s">
+      <c r="B33" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="C33" s="33" t="s">
+      <c r="C33" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="E33" s="32">
+      <c r="E33" s="27">
         <v>2.0</v>
       </c>
-      <c r="F33" s="32">
+      <c r="F33" s="27">
         <v>2.0</v>
       </c>
-      <c r="G33" s="33" t="s">
+      <c r="G33" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="34" ht="30.0" customHeight="1">
-      <c r="A34" s="36" t="s">
+      <c r="A34" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B34" s="36" t="s">
+      <c r="B34" s="25" t="s">
         <v>95</v>
       </c>
-      <c r="C34" s="33" t="s">
+      <c r="C34" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="D34" s="33" t="s">
+      <c r="D34" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="E34" s="32">
+      <c r="E34" s="27">
         <v>1.0</v>
       </c>
-      <c r="F34" s="32">
+      <c r="F34" s="27">
         <v>1.0</v>
       </c>
-      <c r="G34" s="33" t="s">
+      <c r="G34" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="35" ht="30.0" customHeight="1">
-      <c r="A35" s="36" t="s">
+      <c r="A35" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B35" s="36" t="s">
+      <c r="B35" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="C35" s="33" t="s">
+      <c r="C35" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="D35" s="33" t="s">
+      <c r="D35" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="E35" s="32">
+      <c r="E35" s="27">
         <v>1.0</v>
       </c>
-      <c r="F35" s="32">
+      <c r="F35" s="27">
         <v>1.0</v>
       </c>
-      <c r="G35" s="33" t="s">
+      <c r="G35" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="36" ht="30.0" customHeight="1">
-      <c r="A36" s="36" t="s">
+      <c r="A36" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="B36" s="36" t="s">
+      <c r="B36" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="C36" s="33" t="s">
+      <c r="C36" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="D36" s="33" t="s">
+      <c r="D36" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="E36" s="32">
+      <c r="E36" s="27">
         <v>1.0</v>
       </c>
-      <c r="F36" s="32">
+      <c r="F36" s="27">
         <v>1.0</v>
       </c>
-      <c r="G36" s="33" t="s">
+      <c r="G36" s="26" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="37" ht="30.0" customHeight="1">
-      <c r="A37" s="37" t="s">
+      <c r="A37" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="B37" s="37" t="s">
+      <c r="B37" s="30" t="s">
         <v>101</v>
       </c>
-      <c r="C37" s="38" t="s">
+      <c r="C37" s="31" t="s">
         <v>102</v>
       </c>
-      <c r="D37" s="38" t="s">
+      <c r="D37" s="31" t="s">
         <v>68</v>
       </c>
-      <c r="E37" s="39">
+      <c r="E37" s="32">
         <v>1.0</v>
       </c>
-      <c r="F37" s="39">
+      <c r="F37" s="32">
         <v>1.0</v>
       </c>
-      <c r="G37" s="38" t="s">
+      <c r="G37" s="31" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="38" ht="30.0" customHeight="1">
-      <c r="A38" s="40" t="s">
+      <c r="A38" s="33" t="s">
         <v>103</v>
       </c>
-      <c r="B38" s="40" t="s">
+      <c r="B38" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="C38" s="41" t="s">
+      <c r="C38" s="34" t="s">
         <v>105</v>
       </c>
-      <c r="D38" s="41" t="s">
+      <c r="D38" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="E38" s="42">
+      <c r="E38" s="35">
         <v>1.0</v>
       </c>
-      <c r="F38" s="42">
+      <c r="F38" s="35">
         <v>1.0</v>
       </c>
-      <c r="G38" s="41" t="s">
+      <c r="G38" s="34" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="39" ht="30.0" customHeight="1">
-      <c r="A39" s="40" t="s">
+      <c r="A39" s="33" t="s">
         <v>103</v>
       </c>
-      <c r="B39" s="40" t="s">
+      <c r="B39" s="33" t="s">
         <v>106</v>
       </c>
-      <c r="C39" s="41" t="s">
+      <c r="C39" s="34" t="s">
         <v>107</v>
       </c>
-      <c r="D39" s="41" t="s">
+      <c r="D39" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E39" s="42">
+      <c r="E39" s="35">
         <v>1.0</v>
       </c>
-      <c r="F39" s="42">
+      <c r="F39" s="35">
         <v>1.0</v>
       </c>
-      <c r="G39" s="41" t="s">
+      <c r="G39" s="34" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="40" ht="30.0" customHeight="1">
-      <c r="A40" s="40" t="s">
+      <c r="A40" s="33" t="s">
         <v>103</v>
       </c>
-      <c r="B40" s="40" t="s">
+      <c r="B40" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="C40" s="41" t="s">
+      <c r="C40" s="34" t="s">
         <v>109</v>
       </c>
-      <c r="D40" s="41" t="s">
+      <c r="D40" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="E40" s="42">
+      <c r="E40" s="35">
         <v>2.0</v>
       </c>
-      <c r="F40" s="42">
+      <c r="F40" s="35">
         <v>2.0</v>
       </c>
-      <c r="G40" s="41" t="s">
+      <c r="G40" s="34" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="41" ht="30.0" customHeight="1">
-      <c r="A41" s="40" t="s">
+      <c r="A41" s="33" t="s">
         <v>103</v>
       </c>
-      <c r="B41" s="40" t="s">
+      <c r="B41" s="33" t="s">
         <v>110</v>
       </c>
-      <c r="C41" s="41" t="s">
+      <c r="C41" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="D41" s="41" t="s">
+      <c r="D41" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="E41" s="42">
+      <c r="E41" s="35">
         <v>1.0</v>
       </c>
-      <c r="F41" s="42">
+      <c r="F41" s="35">
         <v>1.0</v>
       </c>
-      <c r="G41" s="41" t="s">
+      <c r="G41" s="34" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="42" ht="30.0" customHeight="1">
-      <c r="A42" s="40" t="s">
+      <c r="A42" s="33" t="s">
         <v>103</v>
       </c>
-      <c r="B42" s="40" t="s">
+      <c r="B42" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="C42" s="41" t="s">
+      <c r="C42" s="34" t="s">
         <v>113</v>
       </c>
-      <c r="D42" s="41" t="s">
+      <c r="D42" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="E42" s="42">
+      <c r="E42" s="35">
         <v>2.0</v>
       </c>
-      <c r="F42" s="42">
+      <c r="F42" s="35">
         <v>2.0</v>
       </c>
-      <c r="G42" s="41" t="s">
+      <c r="G42" s="34" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="43" ht="30.0" customHeight="1">
-      <c r="A43" s="40" t="s">
+      <c r="A43" s="33" t="s">
         <v>103</v>
       </c>
-      <c r="B43" s="40" t="s">
+      <c r="B43" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="C43" s="41" t="s">
+      <c r="C43" s="34" t="s">
         <v>115</v>
       </c>
-      <c r="D43" s="41" t="s">
+      <c r="D43" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="E43" s="42">
+      <c r="E43" s="35">
         <v>1.0</v>
       </c>
-      <c r="F43" s="42">
+      <c r="F43" s="35">
         <v>1.0</v>
       </c>
-      <c r="G43" s="41" t="s">
+      <c r="G43" s="34" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="44" ht="30.0" customHeight="1">
-      <c r="A44" s="40" t="s">
+      <c r="A44" s="33" t="s">
         <v>103</v>
       </c>
-      <c r="B44" s="40" t="s">
+      <c r="B44" s="33" t="s">
         <v>116</v>
       </c>
-      <c r="C44" s="41" t="s">
+      <c r="C44" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="D44" s="41" t="s">
+      <c r="D44" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E44" s="42">
+      <c r="E44" s="35">
         <v>1.0</v>
       </c>
-      <c r="F44" s="42">
+      <c r="F44" s="35">
         <v>1.0</v>
       </c>
-      <c r="G44" s="41" t="s">
+      <c r="G44" s="34" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="45" ht="30.0" customHeight="1">
-      <c r="A45" s="43" t="s">
+      <c r="A45" s="36" t="s">
         <v>103</v>
       </c>
-      <c r="B45" s="43" t="s">
+      <c r="B45" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="C45" s="44" t="s">
+      <c r="C45" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="D45" s="45" t="s">
+      <c r="D45" s="38" t="s">
         <v>62</v>
       </c>
-      <c r="E45" s="46">
+      <c r="E45" s="39">
         <v>1.0</v>
       </c>
-      <c r="F45" s="46">
+      <c r="F45" s="39">
         <v>1.0</v>
       </c>
-      <c r="G45" s="44" t="s">
+      <c r="G45" s="37" t="s">
         <v>59</v>
       </c>
-      <c r="H45" s="47"/>
-      <c r="I45" s="47"/>
-      <c r="J45" s="47"/>
-      <c r="K45" s="47"/>
-      <c r="L45" s="47"/>
-      <c r="M45" s="47"/>
-      <c r="N45" s="47"/>
-      <c r="O45" s="47"/>
-      <c r="P45" s="47"/>
-      <c r="Q45" s="47"/>
-      <c r="R45" s="47"/>
-      <c r="S45" s="47"/>
-      <c r="T45" s="47"/>
-      <c r="U45" s="47"/>
-      <c r="V45" s="47"/>
-      <c r="W45" s="47"/>
-      <c r="X45" s="47"/>
-      <c r="Y45" s="47"/>
-      <c r="Z45" s="47"/>
+      <c r="H45" s="40"/>
+      <c r="I45" s="40"/>
+      <c r="J45" s="40"/>
+      <c r="K45" s="40"/>
+      <c r="L45" s="40"/>
+      <c r="M45" s="40"/>
+      <c r="N45" s="40"/>
+      <c r="O45" s="40"/>
+      <c r="P45" s="40"/>
+      <c r="Q45" s="40"/>
+      <c r="R45" s="40"/>
+      <c r="S45" s="40"/>
+      <c r="T45" s="40"/>
+      <c r="U45" s="40"/>
+      <c r="V45" s="40"/>
+      <c r="W45" s="40"/>
+      <c r="X45" s="40"/>
+      <c r="Y45" s="40"/>
+      <c r="Z45" s="40"/>
     </row>
     <row r="46" ht="30.0" customHeight="1">
-      <c r="A46" s="40" t="s">
+      <c r="A46" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="B46" s="40" t="s">
+      <c r="B46" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="C46" s="41" t="s">
+      <c r="C46" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="D46" s="41" t="s">
+      <c r="D46" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="E46" s="42">
+      <c r="E46" s="35">
         <v>2.0</v>
       </c>
-      <c r="F46" s="42">
+      <c r="F46" s="35">
         <v>2.0</v>
       </c>
-      <c r="G46" s="44" t="s">
+      <c r="G46" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="47" ht="30.0" customHeight="1">
-      <c r="A47" s="40" t="s">
+      <c r="A47" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="B47" s="40" t="s">
+      <c r="B47" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="C47" s="41" t="s">
+      <c r="C47" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="D47" s="41" t="s">
+      <c r="D47" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="E47" s="42">
+      <c r="E47" s="35">
         <v>3.0</v>
       </c>
-      <c r="F47" s="42">
+      <c r="F47" s="35">
         <v>3.0</v>
       </c>
-      <c r="G47" s="44" t="s">
+      <c r="G47" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="48" ht="30.0" customHeight="1">
-      <c r="A48" s="40" t="s">
+      <c r="A48" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="B48" s="40" t="s">
+      <c r="B48" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="C48" s="41" t="s">
+      <c r="C48" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="D48" s="41" t="s">
+      <c r="D48" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E48" s="42">
+      <c r="E48" s="35">
         <v>2.0</v>
       </c>
-      <c r="F48" s="42">
+      <c r="F48" s="35">
         <v>2.0</v>
       </c>
-      <c r="G48" s="44" t="s">
+      <c r="G48" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="49" ht="30.0" customHeight="1">
-      <c r="A49" s="40" t="s">
+      <c r="A49" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B49" s="40" t="s">
+      <c r="B49" s="33" t="s">
         <v>128</v>
       </c>
-      <c r="C49" s="41" t="s">
+      <c r="C49" s="34" t="s">
         <v>129</v>
       </c>
-      <c r="D49" s="41" t="s">
+      <c r="D49" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="E49" s="42">
+      <c r="E49" s="35">
         <v>3.0</v>
       </c>
-      <c r="F49" s="42">
+      <c r="F49" s="35">
         <v>3.0</v>
       </c>
-      <c r="G49" s="44" t="s">
+      <c r="G49" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="50" ht="30.0" customHeight="1">
-      <c r="A50" s="40" t="s">
+      <c r="A50" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B50" s="40" t="s">
+      <c r="B50" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="C50" s="41" t="s">
+      <c r="C50" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="D50" s="41" t="s">
+      <c r="D50" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="E50" s="42">
+      <c r="E50" s="35">
         <v>2.0</v>
       </c>
-      <c r="F50" s="42">
+      <c r="F50" s="35">
         <v>2.0</v>
       </c>
-      <c r="G50" s="44" t="s">
+      <c r="G50" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="51" ht="30.0" customHeight="1">
-      <c r="A51" s="40" t="s">
+      <c r="A51" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B51" s="40" t="s">
+      <c r="B51" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="C51" s="41" t="s">
+      <c r="C51" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="D51" s="41" t="s">
+      <c r="D51" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="E51" s="42">
+      <c r="E51" s="35">
         <v>3.0</v>
       </c>
-      <c r="F51" s="42">
+      <c r="F51" s="35">
         <v>3.0</v>
       </c>
-      <c r="G51" s="44" t="s">
+      <c r="G51" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="52" ht="30.0" customHeight="1">
-      <c r="A52" s="40" t="s">
+      <c r="A52" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="B52" s="40" t="s">
+      <c r="B52" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="C52" s="41" t="s">
+      <c r="C52" s="34" t="s">
         <v>136</v>
       </c>
-      <c r="D52" s="41" t="s">
+      <c r="D52" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="E52" s="42">
+      <c r="E52" s="35">
         <v>2.0</v>
       </c>
-      <c r="F52" s="42">
+      <c r="F52" s="35">
         <v>2.0</v>
       </c>
-      <c r="G52" s="44" t="s">
+      <c r="G52" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="53" ht="30.0" customHeight="1">
-      <c r="A53" s="40" t="s">
+      <c r="A53" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="B53" s="40" t="s">
+      <c r="B53" s="33" t="s">
         <v>137</v>
       </c>
-      <c r="C53" s="41" t="s">
+      <c r="C53" s="34" t="s">
         <v>138</v>
       </c>
-      <c r="D53" s="41" t="s">
+      <c r="D53" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="E53" s="42">
+      <c r="E53" s="35">
         <v>2.0</v>
       </c>
-      <c r="F53" s="42">
+      <c r="F53" s="35">
         <v>2.0</v>
       </c>
-      <c r="G53" s="44" t="s">
+      <c r="G53" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="54" ht="30.0" customHeight="1">
-      <c r="A54" s="40" t="s">
+      <c r="A54" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="B54" s="40" t="s">
+      <c r="B54" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="C54" s="41" t="s">
+      <c r="C54" s="34" t="s">
         <v>140</v>
       </c>
-      <c r="D54" s="41" t="s">
+      <c r="D54" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="E54" s="42">
+      <c r="E54" s="35">
         <v>2.0</v>
       </c>
-      <c r="F54" s="42">
+      <c r="F54" s="35">
         <v>2.0</v>
       </c>
-      <c r="G54" s="44" t="s">
+      <c r="G54" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="55" ht="30.0" customHeight="1">
-      <c r="A55" s="40" t="s">
+      <c r="A55" s="33" t="s">
         <v>141</v>
       </c>
-      <c r="B55" s="40" t="s">
+      <c r="B55" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="C55" s="41" t="s">
+      <c r="C55" s="34" t="s">
         <v>143</v>
       </c>
-      <c r="D55" s="41" t="s">
+      <c r="D55" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E55" s="42">
+      <c r="E55" s="35">
         <v>1.0</v>
       </c>
-      <c r="F55" s="42">
+      <c r="F55" s="35">
         <v>1.0</v>
       </c>
-      <c r="G55" s="44" t="s">
+      <c r="G55" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="56" ht="30.0" customHeight="1">
-      <c r="A56" s="40" t="s">
+      <c r="A56" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="B56" s="40" t="s">
+      <c r="B56" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="C56" s="41" t="s">
+      <c r="C56" s="34" t="s">
         <v>146</v>
       </c>
-      <c r="D56" s="41" t="s">
+      <c r="D56" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E56" s="42">
+      <c r="E56" s="35">
         <v>2.0</v>
       </c>
-      <c r="F56" s="42">
+      <c r="F56" s="35">
         <v>2.0</v>
       </c>
-      <c r="G56" s="44" t="s">
+      <c r="G56" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="57" ht="30.0" customHeight="1">
-      <c r="A57" s="40" t="s">
+      <c r="A57" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="B57" s="40" t="s">
+      <c r="B57" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="C57" s="41" t="s">
+      <c r="C57" s="34" t="s">
         <v>149</v>
       </c>
-      <c r="D57" s="41" t="s">
+      <c r="D57" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="E57" s="42">
+      <c r="E57" s="35">
         <v>1.0</v>
       </c>
-      <c r="F57" s="42">
+      <c r="F57" s="35">
         <v>1.0</v>
       </c>
-      <c r="G57" s="44" t="s">
+      <c r="G57" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="58" ht="14.25" customHeight="1">
-      <c r="A58" s="48" t="s">
+      <c r="A58" s="41" t="s">
         <v>150</v>
       </c>
-      <c r="B58" s="49"/>
-      <c r="C58" s="50" t="s">
+      <c r="B58" s="42"/>
+      <c r="C58" s="43" t="s">
         <v>151</v>
       </c>
-      <c r="D58" s="49"/>
-      <c r="E58" s="51">
+      <c r="D58" s="42"/>
+      <c r="E58" s="41">
         <v>36.0</v>
       </c>
-      <c r="F58" s="51">
+      <c r="F58" s="41">
         <v>34.0</v>
       </c>
-      <c r="G58" s="49"/>
+      <c r="G58" s="42"/>
     </row>
     <row r="59" ht="14.25" customHeight="1"/>
     <row r="60" ht="14.25" customHeight="1">
@@ -4642,7 +4640,7 @@
       </c>
     </row>
     <row r="61" ht="14.25" customHeight="1">
-      <c r="A61" s="52" t="s">
+      <c r="A61" s="44" t="s">
         <v>59</v>
       </c>
       <c r="B61" s="9" t="s">
@@ -4650,7 +4648,7 @@
       </c>
     </row>
     <row r="62" ht="14.25" customHeight="1">
-      <c r="A62" s="53" t="s">
+      <c r="A62" s="45" t="s">
         <v>69</v>
       </c>
       <c r="B62" s="9" t="s">
@@ -4658,7 +4656,7 @@
       </c>
     </row>
     <row r="63" ht="14.25" customHeight="1">
-      <c r="A63" s="21" t="s">
+      <c r="A63" s="18" t="s">
         <v>155</v>
       </c>
       <c r="B63" s="9" t="s">
@@ -4666,7 +4664,7 @@
       </c>
     </row>
     <row r="64" ht="14.25" customHeight="1">
-      <c r="A64" s="20" t="s">
+      <c r="A64" s="17" t="s">
         <v>80</v>
       </c>
       <c r="B64" s="9" t="s">
@@ -5662,12 +5660,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="44.25" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="2" ht="14.25" customHeight="1">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="9" t="s">
         <v>159</v>
       </c>
     </row>
@@ -5678,66 +5676,66 @@
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="16" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" ht="27.75" customHeight="1">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="16" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="16" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="16" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="9" ht="30.0" customHeight="1">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="16" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="10" ht="81.0" customHeight="1">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="16" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="16" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B12" s="19" t="s">
+      <c r="B12" s="16" t="s">
         <v>40</v>
       </c>
     </row>
@@ -5759,7 +5757,7 @@
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="17" t="s">
         <v>45</v>
       </c>
       <c r="B16" s="9" t="s">
@@ -5767,7 +5765,7 @@
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="18" t="s">
         <v>47</v>
       </c>
       <c r="B17" s="9" t="s">
@@ -5776,320 +5774,320 @@
     </row>
     <row r="18" ht="14.25" customHeight="1"/>
     <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="22" t="s">
+      <c r="D19" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="F19" s="22" t="s">
+      <c r="F19" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="G19" s="22" t="s">
+      <c r="G19" s="19" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" ht="30.0" customHeight="1">
-      <c r="A20" s="40" t="s">
+      <c r="A20" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="B20" s="40" t="s">
+      <c r="B20" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="C20" s="41" t="s">
+      <c r="C20" s="34" t="s">
         <v>122</v>
       </c>
-      <c r="D20" s="41" t="s">
+      <c r="D20" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="E20" s="42">
+      <c r="E20" s="35">
         <v>2.0</v>
       </c>
-      <c r="F20" s="42">
+      <c r="F20" s="35">
         <v>2.0</v>
       </c>
-      <c r="G20" s="44" t="s">
+      <c r="G20" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="21" ht="30.0" customHeight="1">
-      <c r="A21" s="40" t="s">
+      <c r="A21" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="B21" s="40" t="s">
+      <c r="B21" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="34" t="s">
         <v>124</v>
       </c>
-      <c r="D21" s="41" t="s">
+      <c r="D21" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="E21" s="42">
+      <c r="E21" s="35">
         <v>3.0</v>
       </c>
-      <c r="F21" s="42">
+      <c r="F21" s="35">
         <v>3.0</v>
       </c>
-      <c r="G21" s="44" t="s">
+      <c r="G21" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="22" ht="30.0" customHeight="1">
-      <c r="A22" s="40" t="s">
+      <c r="A22" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="B22" s="40" t="s">
+      <c r="B22" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="C22" s="41" t="s">
+      <c r="C22" s="34" t="s">
         <v>126</v>
       </c>
-      <c r="D22" s="41" t="s">
+      <c r="D22" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E22" s="42">
+      <c r="E22" s="35">
         <v>2.0</v>
       </c>
-      <c r="F22" s="42">
+      <c r="F22" s="35">
         <v>2.0</v>
       </c>
-      <c r="G22" s="44" t="s">
+      <c r="G22" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="23" ht="30.0" customHeight="1">
-      <c r="A23" s="40" t="s">
+      <c r="A23" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B23" s="40" t="s">
+      <c r="B23" s="33" t="s">
         <v>128</v>
       </c>
-      <c r="C23" s="41" t="s">
+      <c r="C23" s="34" t="s">
         <v>129</v>
       </c>
-      <c r="D23" s="41" t="s">
+      <c r="D23" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="E23" s="42">
+      <c r="E23" s="35">
         <v>3.0</v>
       </c>
-      <c r="F23" s="42">
+      <c r="F23" s="35">
         <v>3.0</v>
       </c>
-      <c r="G23" s="44" t="s">
+      <c r="G23" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="24" ht="30.0" customHeight="1">
-      <c r="A24" s="40" t="s">
+      <c r="A24" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B24" s="40" t="s">
+      <c r="B24" s="33" t="s">
         <v>130</v>
       </c>
-      <c r="C24" s="41" t="s">
+      <c r="C24" s="34" t="s">
         <v>131</v>
       </c>
-      <c r="D24" s="41" t="s">
+      <c r="D24" s="34" t="s">
         <v>65</v>
       </c>
-      <c r="E24" s="42">
+      <c r="E24" s="35">
         <v>2.0</v>
       </c>
-      <c r="F24" s="42">
+      <c r="F24" s="35">
         <v>2.0</v>
       </c>
-      <c r="G24" s="44" t="s">
+      <c r="G24" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="25" ht="30.0" customHeight="1">
-      <c r="A25" s="40" t="s">
+      <c r="A25" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="B25" s="40" t="s">
+      <c r="B25" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="C25" s="41" t="s">
+      <c r="C25" s="34" t="s">
         <v>133</v>
       </c>
-      <c r="D25" s="41" t="s">
+      <c r="D25" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="E25" s="42">
+      <c r="E25" s="35">
         <v>3.0</v>
       </c>
-      <c r="F25" s="42">
+      <c r="F25" s="35">
         <v>3.0</v>
       </c>
-      <c r="G25" s="44" t="s">
+      <c r="G25" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="26" ht="30.0" customHeight="1">
-      <c r="A26" s="40" t="s">
+      <c r="A26" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="B26" s="40" t="s">
+      <c r="B26" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="C26" s="41" t="s">
+      <c r="C26" s="34" t="s">
         <v>136</v>
       </c>
-      <c r="D26" s="41" t="s">
+      <c r="D26" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="E26" s="42">
+      <c r="E26" s="35">
         <v>2.0</v>
       </c>
-      <c r="F26" s="42">
+      <c r="F26" s="35">
         <v>2.0</v>
       </c>
-      <c r="G26" s="44" t="s">
+      <c r="G26" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="27" ht="30.0" customHeight="1">
-      <c r="A27" s="40" t="s">
+      <c r="A27" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="B27" s="40" t="s">
+      <c r="B27" s="33" t="s">
         <v>137</v>
       </c>
-      <c r="C27" s="41" t="s">
+      <c r="C27" s="34" t="s">
         <v>138</v>
       </c>
-      <c r="D27" s="41" t="s">
+      <c r="D27" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="E27" s="42">
+      <c r="E27" s="35">
         <v>2.0</v>
       </c>
-      <c r="F27" s="42">
+      <c r="F27" s="35">
         <v>2.0</v>
       </c>
-      <c r="G27" s="44" t="s">
+      <c r="G27" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="28" ht="30.0" customHeight="1">
-      <c r="A28" s="40" t="s">
+      <c r="A28" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="B28" s="40" t="s">
+      <c r="B28" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="C28" s="41" t="s">
+      <c r="C28" s="34" t="s">
         <v>140</v>
       </c>
-      <c r="D28" s="41" t="s">
+      <c r="D28" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="E28" s="42">
+      <c r="E28" s="35">
         <v>2.0</v>
       </c>
-      <c r="F28" s="42">
+      <c r="F28" s="35">
         <v>2.0</v>
       </c>
-      <c r="G28" s="44" t="s">
+      <c r="G28" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="29" ht="30.0" customHeight="1">
-      <c r="A29" s="40" t="s">
+      <c r="A29" s="33" t="s">
         <v>141</v>
       </c>
-      <c r="B29" s="40" t="s">
+      <c r="B29" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="C29" s="41" t="s">
+      <c r="C29" s="34" t="s">
         <v>143</v>
       </c>
-      <c r="D29" s="41" t="s">
+      <c r="D29" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E29" s="42">
+      <c r="E29" s="35">
         <v>1.0</v>
       </c>
-      <c r="F29" s="42">
+      <c r="F29" s="35">
         <v>1.0</v>
       </c>
-      <c r="G29" s="44" t="s">
+      <c r="G29" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="30" ht="30.0" customHeight="1">
-      <c r="A30" s="40" t="s">
+      <c r="A30" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="B30" s="40" t="s">
+      <c r="B30" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="C30" s="41" t="s">
+      <c r="C30" s="34" t="s">
         <v>146</v>
       </c>
-      <c r="D30" s="41" t="s">
+      <c r="D30" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="42">
+      <c r="E30" s="35">
         <v>2.0</v>
       </c>
-      <c r="F30" s="42">
+      <c r="F30" s="35">
         <v>2.0</v>
       </c>
-      <c r="G30" s="44" t="s">
+      <c r="G30" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="31" ht="30.0" customHeight="1">
-      <c r="A31" s="40" t="s">
+      <c r="A31" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="B31" s="40" t="s">
+      <c r="B31" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="C31" s="41" t="s">
+      <c r="C31" s="34" t="s">
         <v>149</v>
       </c>
-      <c r="D31" s="41" t="s">
+      <c r="D31" s="34" t="s">
         <v>62</v>
       </c>
-      <c r="E31" s="42">
+      <c r="E31" s="35">
         <v>1.0</v>
       </c>
-      <c r="F31" s="42">
+      <c r="F31" s="35">
         <v>1.0</v>
       </c>
-      <c r="G31" s="44" t="s">
+      <c r="G31" s="37" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="32" ht="14.25" customHeight="1">
-      <c r="A32" s="48" t="s">
+      <c r="A32" s="41" t="s">
         <v>150</v>
       </c>
-      <c r="B32" s="49"/>
-      <c r="C32" s="50" t="s">
+      <c r="B32" s="42"/>
+      <c r="C32" s="43" t="s">
         <v>162</v>
       </c>
-      <c r="D32" s="49"/>
-      <c r="E32" s="51">
+      <c r="D32" s="42"/>
+      <c r="E32" s="41">
         <v>25.0</v>
       </c>
-      <c r="F32" s="51">
+      <c r="F32" s="41">
         <v>25.0</v>
       </c>
-      <c r="G32" s="49"/>
+      <c r="G32" s="42"/>
     </row>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1">
@@ -6098,7 +6096,7 @@
       </c>
     </row>
     <row r="35" ht="14.25" customHeight="1">
-      <c r="A35" s="52" t="s">
+      <c r="A35" s="44" t="s">
         <v>59</v>
       </c>
       <c r="B35" s="9" t="s">
@@ -6106,7 +6104,7 @@
       </c>
     </row>
     <row r="36" ht="14.25" customHeight="1">
-      <c r="A36" s="53" t="s">
+      <c r="A36" s="45" t="s">
         <v>69</v>
       </c>
       <c r="B36" s="9" t="s">
@@ -6114,7 +6112,7 @@
       </c>
     </row>
     <row r="37" ht="14.25" customHeight="1">
-      <c r="A37" s="21" t="s">
+      <c r="A37" s="18" t="s">
         <v>155</v>
       </c>
       <c r="B37" s="9" t="s">
@@ -6122,7 +6120,7 @@
       </c>
     </row>
     <row r="38" ht="14.25" customHeight="1">
-      <c r="A38" s="20" t="s">
+      <c r="A38" s="17" t="s">
         <v>80</v>
       </c>
       <c r="B38" s="9" t="s">
@@ -7115,8 +7113,8 @@
     <col customWidth="1" min="6" max="26" width="8.86"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1">
-      <c r="A1" s="54" t="s">
+    <row r="1" ht="58.5" customHeight="1">
+      <c r="A1" s="14" t="s">
         <v>163</v>
       </c>
     </row>
@@ -7138,163 +7136,259 @@
       <c r="A5" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="9" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="6" ht="14.25" customHeight="1"/>
     <row r="7" ht="14.25" customHeight="1">
-      <c r="A7" s="55" t="s">
+      <c r="A7" s="46" t="s">
         <v>169</v>
       </c>
-      <c r="B7" s="55" t="s">
+      <c r="B7" s="46" t="s">
         <v>170</v>
       </c>
-      <c r="C7" s="55" t="s">
+      <c r="C7" s="46" t="s">
         <v>171</v>
       </c>
-      <c r="D7" s="55" t="s">
+      <c r="D7" s="46" t="s">
         <v>172</v>
       </c>
-      <c r="E7" s="55" t="s">
+      <c r="E7" s="46" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="8" ht="24.75" customHeight="1">
-      <c r="A8" s="56" t="s">
+      <c r="A8" s="47" t="s">
         <v>174</v>
       </c>
-      <c r="B8" s="57">
+      <c r="B8" s="48">
+        <v>36.0</v>
+      </c>
+      <c r="C8" s="48">
+        <v>36.0</v>
+      </c>
+      <c r="D8" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="9" ht="24.75" customHeight="1">
+      <c r="A9" s="47" t="s">
+        <v>176</v>
+      </c>
+      <c r="B9" s="48">
+        <v>27.0</v>
+      </c>
+      <c r="C9" s="48">
+        <v>27.0</v>
+      </c>
+      <c r="D9" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="10" ht="24.75" customHeight="1">
+      <c r="A10" s="47" t="s">
+        <v>178</v>
+      </c>
+      <c r="B10" s="48">
         <v>18.0</v>
       </c>
-      <c r="C8" s="57">
+      <c r="C10" s="48">
         <v>18.0</v>
       </c>
-      <c r="D8" s="57">
+      <c r="D10" s="48">
         <v>0.0</v>
       </c>
-      <c r="E8" s="19" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="9" ht="24.75" customHeight="1">
-      <c r="A9" s="56" t="s">
-        <v>176</v>
-      </c>
-      <c r="B9" s="57">
-        <v>13.5</v>
-      </c>
-      <c r="C9" s="57" t="s">
-        <v>177</v>
-      </c>
-      <c r="D9" s="57"/>
-      <c r="E9" s="19" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" ht="24.75" customHeight="1">
-      <c r="A10" s="56" t="s">
+      <c r="E10" s="16" t="s">
         <v>179</v>
       </c>
-      <c r="B10" s="57">
+    </row>
+    <row r="11" ht="24.75" customHeight="1">
+      <c r="A11" s="47" t="s">
+        <v>180</v>
+      </c>
+      <c r="B11" s="48">
         <v>9.0</v>
       </c>
-      <c r="C10" s="57" t="s">
-        <v>177</v>
-      </c>
-      <c r="D10" s="57"/>
-      <c r="E10" s="19" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="11" ht="24.75" customHeight="1">
-      <c r="A11" s="56" t="s">
+      <c r="C11" s="48">
+        <v>9.0</v>
+      </c>
+      <c r="D11" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="E11" s="16" t="s">
         <v>181</v>
       </c>
-      <c r="B11" s="57">
-        <v>4.5</v>
-      </c>
-      <c r="C11" s="57" t="s">
-        <v>177</v>
-      </c>
-      <c r="D11" s="57"/>
-      <c r="E11" s="19" t="s">
+    </row>
+    <row r="12" ht="24.75" customHeight="1">
+      <c r="A12" s="47" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="12" ht="24.75" customHeight="1">
-      <c r="A12" s="56" t="s">
+      <c r="B12" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="C12" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="D12" s="48">
+        <v>0.0</v>
+      </c>
+      <c r="E12" s="16" t="s">
         <v>183</v>
-      </c>
-      <c r="B12" s="57">
-        <v>0.0</v>
-      </c>
-      <c r="C12" s="57" t="s">
-        <v>177</v>
-      </c>
-      <c r="D12" s="57"/>
-      <c r="E12" s="19" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1"/>
     <row r="14" ht="14.25" customHeight="1"/>
     <row r="15" ht="14.25" customHeight="1">
       <c r="A15" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B15" s="7" t="s">
         <v>185</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1"/>
     <row r="17" ht="14.25" customHeight="1">
       <c r="A17" s="3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="18" ht="14.25" customHeight="1">
+      <c r="A18" s="17" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="18" ht="14.25" customHeight="1">
-      <c r="A18" s="20" t="s">
+      <c r="B18" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="B18" s="9" t="s">
+    </row>
+    <row r="19" ht="14.25" customHeight="1">
+      <c r="A19" s="45" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="19" ht="14.25" customHeight="1">
-      <c r="A19" s="53" t="s">
+      <c r="B19" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="B19" s="9" t="s">
+    </row>
+    <row r="20" ht="14.25" customHeight="1">
+      <c r="A20" s="17" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="20" ht="14.25" customHeight="1">
-      <c r="A20" s="20" t="s">
+      <c r="B20" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="B20" s="9" t="s">
+    </row>
+    <row r="21" ht="14.25" customHeight="1">
+      <c r="A21" s="18" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="21" ht="14.25" customHeight="1">
-      <c r="A21" s="21" t="s">
+      <c r="B21" s="9" t="s">
         <v>194</v>
       </c>
-      <c r="B21" s="9" t="s">
+    </row>
+    <row r="22" ht="14.25" customHeight="1"/>
+    <row r="23" ht="14.25" customHeight="1">
+      <c r="A23" s="49" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="22" ht="14.25" customHeight="1"/>
-    <row r="23" ht="14.25" customHeight="1"/>
     <row r="24" ht="14.25" customHeight="1"/>
     <row r="25" ht="14.25" customHeight="1"/>
-    <row r="26" ht="14.25" customHeight="1"/>
-    <row r="27" ht="14.25" customHeight="1"/>
-    <row r="28" ht="14.25" customHeight="1"/>
-    <row r="29" ht="14.25" customHeight="1"/>
-    <row r="30" ht="14.25" customHeight="1"/>
-    <row r="31" ht="14.25" customHeight="1"/>
+    <row r="26" ht="14.25" customHeight="1">
+      <c r="A26" s="50" t="s">
+        <v>196</v>
+      </c>
+      <c r="B26" s="50" t="s">
+        <v>197</v>
+      </c>
+      <c r="C26" s="50" t="s">
+        <v>198</v>
+      </c>
+      <c r="D26" s="50" t="s">
+        <v>199</v>
+      </c>
+      <c r="E26" s="51"/>
+    </row>
+    <row r="27" ht="39.0" customHeight="1">
+      <c r="A27" s="52" t="s">
+        <v>174</v>
+      </c>
+      <c r="B27" s="53">
+        <v>0.0</v>
+      </c>
+      <c r="C27" s="53">
+        <v>0.0</v>
+      </c>
+      <c r="D27" s="53">
+        <v>36.0</v>
+      </c>
+      <c r="E27" s="54"/>
+    </row>
+    <row r="28" ht="36.75" customHeight="1">
+      <c r="A28" s="52" t="s">
+        <v>176</v>
+      </c>
+      <c r="B28" s="53">
+        <v>9.0</v>
+      </c>
+      <c r="C28" s="53">
+        <v>9.0</v>
+      </c>
+      <c r="D28" s="53">
+        <v>36.0</v>
+      </c>
+      <c r="E28" s="54"/>
+    </row>
+    <row r="29" ht="30.75" customHeight="1">
+      <c r="A29" s="52" t="s">
+        <v>178</v>
+      </c>
+      <c r="B29" s="53">
+        <v>18.0</v>
+      </c>
+      <c r="C29" s="53">
+        <v>18.0</v>
+      </c>
+      <c r="D29" s="53">
+        <v>36.0</v>
+      </c>
+      <c r="E29" s="54"/>
+    </row>
+    <row r="30" ht="30.0" customHeight="1">
+      <c r="A30" s="52" t="s">
+        <v>180</v>
+      </c>
+      <c r="B30" s="53">
+        <v>27.0</v>
+      </c>
+      <c r="C30" s="53">
+        <v>27.0</v>
+      </c>
+      <c r="D30" s="53">
+        <v>36.0</v>
+      </c>
+      <c r="E30" s="54"/>
+    </row>
+    <row r="31" ht="48.0" customHeight="1">
+      <c r="A31" s="52" t="s">
+        <v>182</v>
+      </c>
+      <c r="B31" s="53">
+        <v>36.0</v>
+      </c>
+      <c r="C31" s="53">
+        <v>36.0</v>
+      </c>
+      <c r="D31" s="53">
+        <v>36.0</v>
+      </c>
+      <c r="E31" s="54"/>
+    </row>
     <row r="32" ht="14.25" customHeight="1"/>
     <row r="33" ht="14.25" customHeight="1"/>
     <row r="34" ht="14.25" customHeight="1"/>
@@ -8289,135 +8383,135 @@
     <row r="1" ht="14.25" customHeight="1"/>
     <row r="2" ht="14.25" customHeight="1">
       <c r="B2" s="2" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="B3" s="9" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="4" ht="14.25" customHeight="1"/>
     <row r="5" ht="14.25" customHeight="1">
-      <c r="A5" s="55"/>
-      <c r="B5" s="55" t="s">
-        <v>198</v>
-      </c>
-      <c r="C5" s="55" t="s">
-        <v>199</v>
-      </c>
-      <c r="D5" s="58" t="s">
-        <v>200</v>
+      <c r="A5" s="46"/>
+      <c r="B5" s="46" t="s">
+        <v>202</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>203</v>
+      </c>
+      <c r="D5" s="55" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="6" ht="30.0" customHeight="1">
-      <c r="B6" s="59" t="s">
-        <v>201</v>
-      </c>
-      <c r="C6" s="60" t="s">
-        <v>202</v>
-      </c>
-      <c r="D6" s="59" t="s">
-        <v>203</v>
+      <c r="B6" s="56" t="s">
+        <v>205</v>
+      </c>
+      <c r="C6" s="57" t="s">
+        <v>206</v>
+      </c>
+      <c r="D6" s="56" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="7" ht="30.0" customHeight="1">
-      <c r="B7" s="59" t="s">
-        <v>204</v>
-      </c>
-      <c r="C7" s="60" t="s">
-        <v>205</v>
-      </c>
-      <c r="D7" s="59" t="s">
-        <v>206</v>
+      <c r="B7" s="56" t="s">
+        <v>208</v>
+      </c>
+      <c r="C7" s="57" t="s">
+        <v>209</v>
+      </c>
+      <c r="D7" s="56" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="8" ht="30.0" customHeight="1">
-      <c r="B8" s="59" t="s">
-        <v>207</v>
-      </c>
-      <c r="C8" s="60" t="s">
-        <v>208</v>
-      </c>
-      <c r="D8" s="59" t="s">
+      <c r="B8" s="56" t="s">
+        <v>211</v>
+      </c>
+      <c r="C8" s="57" t="s">
+        <v>212</v>
+      </c>
+      <c r="D8" s="56" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="9" ht="30.0" customHeight="1">
+      <c r="B9" s="56" t="s">
+        <v>214</v>
+      </c>
+      <c r="C9" s="57" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="9" ht="30.0" customHeight="1">
-      <c r="B9" s="59" t="s">
-        <v>210</v>
-      </c>
-      <c r="C9" s="60" t="s">
-        <v>205</v>
-      </c>
-      <c r="D9" s="59" t="s">
-        <v>211</v>
+      <c r="D9" s="56" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="10" ht="30.0" customHeight="1">
-      <c r="B10" s="59" t="s">
-        <v>212</v>
-      </c>
-      <c r="C10" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="D10" s="59" t="s">
-        <v>214</v>
+      <c r="B10" s="56" t="s">
+        <v>216</v>
+      </c>
+      <c r="C10" s="57" t="s">
+        <v>217</v>
+      </c>
+      <c r="D10" s="56" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="11" ht="30.0" customHeight="1">
-      <c r="B11" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="C11" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="D11" s="61" t="s">
-        <v>216</v>
+      <c r="B11" s="56" t="s">
+        <v>219</v>
+      </c>
+      <c r="C11" s="57" t="s">
+        <v>217</v>
+      </c>
+      <c r="D11" s="56" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="12" ht="30.0" customHeight="1">
-      <c r="B12" s="59" t="s">
+      <c r="B12" s="56" t="s">
+        <v>221</v>
+      </c>
+      <c r="C12" s="57" t="s">
         <v>217</v>
       </c>
-      <c r="C12" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="D12" s="59" t="s">
-        <v>218</v>
+      <c r="D12" s="56" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="13" ht="30.0" customHeight="1">
-      <c r="B13" s="59" t="s">
-        <v>219</v>
-      </c>
-      <c r="C13" s="60" t="s">
-        <v>220</v>
-      </c>
-      <c r="D13" s="59" t="s">
-        <v>221</v>
+      <c r="B13" s="56" t="s">
+        <v>223</v>
+      </c>
+      <c r="C13" s="57" t="s">
+        <v>224</v>
+      </c>
+      <c r="D13" s="56" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="14" ht="30.0" customHeight="1">
-      <c r="B14" s="59" t="s">
-        <v>222</v>
-      </c>
-      <c r="C14" s="60" t="s">
-        <v>213</v>
-      </c>
-      <c r="D14" s="59" t="s">
-        <v>223</v>
+      <c r="B14" s="56" t="s">
+        <v>226</v>
+      </c>
+      <c r="C14" s="57" t="s">
+        <v>217</v>
+      </c>
+      <c r="D14" s="56" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="15" ht="30.0" customHeight="1">
-      <c r="B15" s="59" t="s">
-        <v>224</v>
-      </c>
-      <c r="C15" s="62" t="s">
-        <v>225</v>
-      </c>
-      <c r="D15" s="59" t="s">
-        <v>226</v>
+      <c r="B15" s="56" t="s">
+        <v>228</v>
+      </c>
+      <c r="C15" s="57" t="s">
+        <v>229</v>
+      </c>
+      <c r="D15" s="56" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="16" ht="14.25" customHeight="1"/>

</xml_diff>